<commit_message>
Add intraday research observations and selectable Excel watchlists
</commit_message>
<xml_diff>
--- a/dashboard/excel_numeric/template.xlsx
+++ b/dashboard/excel_numeric/template.xlsx
@@ -2,14 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数字看板" sheetId="1" r:id="Rb9bc0ffcf7ed49d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分位与样本" sheetId="2" r:id="Rc7d2b67af08641a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="研究指标" sheetId="3" r:id="R686106b137e34d85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与状态" sheetId="4" r:id="Rac62a8c3fb304e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡片数据" sheetId="5" r:id="R0a571c47ccc54ecc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标数据" sheetId="6" r:id="R91fef455b2354fa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="7" r:id="R5bcce115fb0f4096"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标" sheetId="8" r:id="R153e38adb15a4028"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数字看板" sheetId="1" r:id="Rf771bce119a04772"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分位与样本" sheetId="2" r:id="R046f2abfd4584d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="研究指标" sheetId="3" r:id="R45ffa40df11348b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源与状态" sheetId="4" r:id="R60e3124ca3174045"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="卡片数据" sheetId="5" r:id="R62388c5cfc5e4dfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标数据" sheetId="6" r:id="R877762f2ccee4ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="概览" sheetId="7" r:id="Ref6abc7999a24194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="指标" sheetId="8" r:id="Rc444f5ed87f745e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="组合对比" sheetId="9" r:id="R2da7ff3009bc4f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="合约选项" sheetId="10" r:id="R3be22be7f2ec4fd1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +22,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="12">
+  <x:numFmts count="14">
     <x:numFmt numFmtId="200" formatCode="0.0000"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="0.0000%"/>
@@ -33,8 +35,10 @@
     <x:numFmt numFmtId="209" formatCode="0%"/>
     <x:numFmt numFmtId="210" formatCode="&quot;n=&quot;0"/>
     <x:numFmt numFmtId="211" formatCode="mm/dd hh:mm"/>
+    <x:numFmt numFmtId="212" formatCode="mm/dd hh:mm:ss"/>
+    <x:numFmt numFmtId="213" formatCode="mm/dd"/>
   </x:numFmts>
-  <x:fonts count="15">
+  <x:fonts count="18">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -104,12 +108,28 @@
       <x:name val="Microsoft YaHei"/>
     </x:font>
     <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF203348"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
       <x:sz val="10"/>
       <x:color rgb="FF64748B"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
     <x:font>
-      <x:sz val="11"/>
+      <x:sz val="10"/>
+      <x:color rgb="FF087E8B"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
@@ -154,7 +174,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="51">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -249,8 +269,11 @@
     <x:xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="205" fontId="13" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="205" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -258,7 +281,7 @@
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="205" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -281,6 +304,64 @@
     </x:xf>
     <x:xf numFmtId="211" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="14" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="208" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="212" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="213" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -431,7 +512,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R002f768ad5694e87"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Racdf5a46c3f54e3b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1970,6 +2051,20 @@
 </x:worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>具体合约与指数</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
@@ -24159,10 +24254,10 @@
     <x:row r="12" ht="19" customHeight="1">
       <x:c r="A12" s="14"/>
       <x:c r="B12" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="C12" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="D12" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!L$7:L$406,$E$3*4+1)),"",INDEX('卡片数据'!L$7:L$406,$E$3*4+1))</x:f>
@@ -24180,10 +24275,10 @@
       <x:c r="I12" s="33"/>
       <x:c r="J12" s="14"/>
       <x:c r="K12" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="L12" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="M12" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!L$7:L$406,$E$3*4+2)),"",INDEX('卡片数据'!L$7:L$406,$E$3*4+2))</x:f>
@@ -24349,29 +24444,29 @@
       <x:c r="R16" s="37"/>
       <x:c r="S16" s="14"/>
     </x:row>
-    <x:row r="17" ht="19" customHeight="1">
+    <x:row r="17" ht="30" customHeight="1">
       <x:c r="A17" s="14"/>
-      <x:c r="B17" s="40" t="str">
+      <x:c r="B17" s="41" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!V$7:V$406,$E$3*4+1)),"",INDEX('卡片数据'!V$7:V$406,$E$3*4+1))</x:f>
       </x:c>
-      <x:c r="C17" s="40"/>
-      <x:c r="D17" s="40"/>
-      <x:c r="E17" s="40"/>
-      <x:c r="F17" s="40"/>
-      <x:c r="G17" s="40"/>
-      <x:c r="H17" s="40"/>
-      <x:c r="I17" s="40"/>
+      <x:c r="C17" s="41"/>
+      <x:c r="D17" s="41"/>
+      <x:c r="E17" s="41"/>
+      <x:c r="F17" s="41"/>
+      <x:c r="G17" s="41"/>
+      <x:c r="H17" s="41"/>
+      <x:c r="I17" s="41"/>
       <x:c r="J17" s="14"/>
-      <x:c r="K17" s="40" t="str">
+      <x:c r="K17" s="41" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!V$7:V$406,$E$3*4+2)),"",INDEX('卡片数据'!V$7:V$406,$E$3*4+2))</x:f>
       </x:c>
-      <x:c r="L17" s="40"/>
-      <x:c r="M17" s="40"/>
-      <x:c r="N17" s="40"/>
-      <x:c r="O17" s="40"/>
-      <x:c r="P17" s="40"/>
-      <x:c r="Q17" s="40"/>
-      <x:c r="R17" s="40"/>
+      <x:c r="L17" s="41"/>
+      <x:c r="M17" s="41"/>
+      <x:c r="N17" s="41"/>
+      <x:c r="O17" s="41"/>
+      <x:c r="P17" s="41"/>
+      <x:c r="Q17" s="41"/>
+      <x:c r="R17" s="41"/>
       <x:c r="S17" s="14"/>
     </x:row>
     <x:row r="18" ht="19" customHeight="1">
@@ -24642,10 +24737,10 @@
     <x:row r="25" ht="19" customHeight="1">
       <x:c r="A25" s="14"/>
       <x:c r="B25" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="C25" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="D25" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!L$7:L$406,$E$3*4+3)),"",INDEX('卡片数据'!L$7:L$406,$E$3*4+3))</x:f>
@@ -24663,10 +24758,10 @@
       <x:c r="I25" s="33"/>
       <x:c r="J25" s="14"/>
       <x:c r="K25" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="L25" s="31" t="str">
-        <x:v>日换手 倍</x:v>
+        <x:v>换手 倍</x:v>
       </x:c>
       <x:c r="M25" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!L$7:L$406,$E$3*4+4)),"",INDEX('卡片数据'!L$7:L$406,$E$3*4+4))</x:f>
@@ -24832,29 +24927,29 @@
       <x:c r="R29" s="37"/>
       <x:c r="S29" s="14"/>
     </x:row>
-    <x:row r="30" ht="19" customHeight="1">
+    <x:row r="30" ht="30" customHeight="1">
       <x:c r="A30" s="14"/>
-      <x:c r="B30" s="40" t="str">
+      <x:c r="B30" s="41" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!V$7:V$406,$E$3*4+3)),"",INDEX('卡片数据'!V$7:V$406,$E$3*4+3))</x:f>
       </x:c>
-      <x:c r="C30" s="40"/>
-      <x:c r="D30" s="40"/>
-      <x:c r="E30" s="40"/>
-      <x:c r="F30" s="40"/>
-      <x:c r="G30" s="40"/>
-      <x:c r="H30" s="40"/>
-      <x:c r="I30" s="40"/>
+      <x:c r="C30" s="41"/>
+      <x:c r="D30" s="41"/>
+      <x:c r="E30" s="41"/>
+      <x:c r="F30" s="41"/>
+      <x:c r="G30" s="41"/>
+      <x:c r="H30" s="41"/>
+      <x:c r="I30" s="41"/>
       <x:c r="J30" s="14"/>
-      <x:c r="K30" s="40" t="str">
+      <x:c r="K30" s="41" t="str">
         <x:f>IF(ISBLANK(INDEX('卡片数据'!V$7:V$406,$E$3*4+4)),"",INDEX('卡片数据'!V$7:V$406,$E$3*4+4))</x:f>
       </x:c>
-      <x:c r="L30" s="40"/>
-      <x:c r="M30" s="40"/>
-      <x:c r="N30" s="40"/>
-      <x:c r="O30" s="40"/>
-      <x:c r="P30" s="40"/>
-      <x:c r="Q30" s="40"/>
-      <x:c r="R30" s="40"/>
+      <x:c r="L30" s="41"/>
+      <x:c r="M30" s="41"/>
+      <x:c r="N30" s="41"/>
+      <x:c r="O30" s="41"/>
+      <x:c r="P30" s="41"/>
+      <x:c r="Q30" s="41"/>
+      <x:c r="R30" s="41"/>
       <x:c r="S30" s="14"/>
     </x:row>
     <x:row r="31" ht="19" customHeight="1">
@@ -25069,110 +25164,110 @@
     </x:row>
     <x:row r="41" ht="19" customHeight="1">
       <x:c r="A41" s="14"/>
-      <x:c r="B41" s="41" t="str">
+      <x:c r="B41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="C41" s="41" t="str">
+      <x:c r="C41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="D41" s="41" t="str">
+      <x:c r="D41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="E41" s="41" t="str">
+      <x:c r="E41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="F41" s="41" t="str">
+      <x:c r="F41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="G41" s="41" t="str">
+      <x:c r="G41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="H41" s="41" t="str">
+      <x:c r="H41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="I41" s="41" t="str">
+      <x:c r="I41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="J41" s="41" t="str">
+      <x:c r="J41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="K41" s="41" t="str">
+      <x:c r="K41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="L41" s="41" t="str">
+      <x:c r="L41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="M41" s="41" t="str">
+      <x:c r="M41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="N41" s="41" t="str">
+      <x:c r="N41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="O41" s="41" t="str">
+      <x:c r="O41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="P41" s="41" t="str">
+      <x:c r="P41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="Q41" s="41" t="str">
+      <x:c r="Q41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="R41" s="41" t="str">
+      <x:c r="R41" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
       <x:c r="S41" s="14"/>
     </x:row>
     <x:row r="42" ht="19" customHeight="1">
       <x:c r="A42" s="14"/>
-      <x:c r="B42" s="41" t="str">
+      <x:c r="B42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="C42" s="41" t="str">
+      <x:c r="C42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="D42" s="41" t="str">
+      <x:c r="D42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="E42" s="41" t="str">
+      <x:c r="E42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="F42" s="41" t="str">
+      <x:c r="F42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="G42" s="41" t="str">
+      <x:c r="G42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="H42" s="41" t="str">
+      <x:c r="H42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="I42" s="41" t="str">
+      <x:c r="I42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="J42" s="41" t="str">
+      <x:c r="J42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="K42" s="41" t="str">
+      <x:c r="K42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="L42" s="41" t="str">
+      <x:c r="L42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="M42" s="41" t="str">
+      <x:c r="M42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="N42" s="41" t="str">
+      <x:c r="N42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="O42" s="41" t="str">
+      <x:c r="O42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="P42" s="41" t="str">
+      <x:c r="P42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="Q42" s="41" t="str">
+      <x:c r="Q42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
-      <x:c r="R42" s="41" t="str">
+      <x:c r="R42" s="42" t="str">
         <x:v>计算 / 写入 / 保存：待完成</x:v>
       </x:c>
       <x:c r="S42" s="14"/>
@@ -25378,7 +25473,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4f3a6cefbf44ef7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7b9ded626cc1408b"/>
 </x:worksheet>
 </file>
 
@@ -25581,46 +25676,46 @@
     </x:row>
     <x:row r="6" ht="27" customHeight="1">
       <x:c r="A6" s="14"/>
-      <x:c r="B6" s="43" t="str">
+      <x:c r="B6" s="44" t="str">
         <x:v>指标</x:v>
       </x:c>
-      <x:c r="C6" s="43" t="str">
+      <x:c r="C6" s="44" t="str">
         <x:v>单位</x:v>
       </x:c>
-      <x:c r="D6" s="43" t="str">
+      <x:c r="D6" s="44" t="str">
         <x:v>IF</x:v>
       </x:c>
-      <x:c r="E6" s="43" t="str">
+      <x:c r="E6" s="44" t="str">
         <x:v>数据时间</x:v>
       </x:c>
-      <x:c r="F6" s="43" t="str">
+      <x:c r="F6" s="44" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="G6" s="43" t="str">
+      <x:c r="G6" s="44" t="str">
         <x:v>IH</x:v>
       </x:c>
-      <x:c r="H6" s="43" t="str">
+      <x:c r="H6" s="44" t="str">
         <x:v>数据时间</x:v>
       </x:c>
-      <x:c r="I6" s="43" t="str">
+      <x:c r="I6" s="44" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="J6" s="43" t="str">
+      <x:c r="J6" s="44" t="str">
         <x:v>IC</x:v>
       </x:c>
-      <x:c r="K6" s="43" t="str">
+      <x:c r="K6" s="44" t="str">
         <x:v>数据时间</x:v>
       </x:c>
-      <x:c r="L6" s="43" t="str">
+      <x:c r="L6" s="44" t="str">
         <x:v>状态</x:v>
       </x:c>
-      <x:c r="M6" s="43" t="str">
+      <x:c r="M6" s="44" t="str">
         <x:v>IM</x:v>
       </x:c>
-      <x:c r="N6" s="43" t="str">
+      <x:c r="N6" s="44" t="str">
         <x:v>数据时间</x:v>
       </x:c>
-      <x:c r="O6" s="43" t="str">
+      <x:c r="O6" s="44" t="str">
         <x:v>状态</x:v>
       </x:c>
       <x:c r="P6" s="14"/>
@@ -25636,7 +25731,7 @@
       <x:c r="D7" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+1)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+1))</x:f>
       </x:c>
-      <x:c r="E7" s="50" t="str">
+      <x:c r="E7" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+1)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+1))</x:f>
       </x:c>
       <x:c r="F7" s="23" t="str">
@@ -25645,7 +25740,7 @@
       <x:c r="G7" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+1)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+1))</x:f>
       </x:c>
-      <x:c r="H7" s="50" t="str">
+      <x:c r="H7" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+1)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+1))</x:f>
       </x:c>
       <x:c r="I7" s="23" t="str">
@@ -25654,7 +25749,7 @@
       <x:c r="J7" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+1)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+1))</x:f>
       </x:c>
-      <x:c r="K7" s="50" t="str">
+      <x:c r="K7" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+1)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+1))</x:f>
       </x:c>
       <x:c r="L7" s="23" t="str">
@@ -25663,7 +25758,7 @@
       <x:c r="M7" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+1)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+1))</x:f>
       </x:c>
-      <x:c r="N7" s="50" t="str">
+      <x:c r="N7" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+1)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+1))</x:f>
       </x:c>
       <x:c r="O7" s="23" t="str">
@@ -25676,43 +25771,43 @@
       <x:c r="B8" s="14" t="str">
         <x:v>调整基差</x:v>
       </x:c>
-      <x:c r="C8" s="45" t="str">
+      <x:c r="C8" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+2)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="D8" s="47" t="str">
+      <x:c r="D8" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+2)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="E8" s="49" t="str">
+      <x:c r="E8" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+2)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="F8" s="45" t="str">
+      <x:c r="F8" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+2)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="G8" s="47" t="str">
+      <x:c r="G8" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+2)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="H8" s="49" t="str">
+      <x:c r="H8" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+2)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="I8" s="45" t="str">
+      <x:c r="I8" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+2)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="J8" s="47" t="str">
+      <x:c r="J8" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+2)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="K8" s="49" t="str">
+      <x:c r="K8" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+2)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="L8" s="45" t="str">
+      <x:c r="L8" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+2)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="M8" s="47" t="str">
+      <x:c r="M8" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+2)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="N8" s="49" t="str">
+      <x:c r="N8" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+2)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+2))</x:f>
       </x:c>
-      <x:c r="O8" s="45" t="str">
+      <x:c r="O8" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+2)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+2))</x:f>
       </x:c>
       <x:c r="P8" s="14"/>
@@ -25728,7 +25823,7 @@
       <x:c r="D9" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+3)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+3))</x:f>
       </x:c>
-      <x:c r="E9" s="50" t="str">
+      <x:c r="E9" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+3)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+3))</x:f>
       </x:c>
       <x:c r="F9" s="23" t="str">
@@ -25737,7 +25832,7 @@
       <x:c r="G9" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+3)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+3))</x:f>
       </x:c>
-      <x:c r="H9" s="50" t="str">
+      <x:c r="H9" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+3)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+3))</x:f>
       </x:c>
       <x:c r="I9" s="23" t="str">
@@ -25746,7 +25841,7 @@
       <x:c r="J9" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+3)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+3))</x:f>
       </x:c>
-      <x:c r="K9" s="50" t="str">
+      <x:c r="K9" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+3)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+3))</x:f>
       </x:c>
       <x:c r="L9" s="23" t="str">
@@ -25755,7 +25850,7 @@
       <x:c r="M9" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+3)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+3))</x:f>
       </x:c>
-      <x:c r="N9" s="50" t="str">
+      <x:c r="N9" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+3)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+3))</x:f>
       </x:c>
       <x:c r="O9" s="23" t="str">
@@ -25768,43 +25863,43 @@
       <x:c r="B10" s="14" t="str">
         <x:v>每日收敛</x:v>
       </x:c>
-      <x:c r="C10" s="45" t="str">
+      <x:c r="C10" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+4)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="D10" s="47" t="str">
+      <x:c r="D10" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+4)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="E10" s="49" t="str">
+      <x:c r="E10" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+4)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="F10" s="45" t="str">
+      <x:c r="F10" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+4)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="G10" s="47" t="str">
+      <x:c r="G10" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+4)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="H10" s="49" t="str">
+      <x:c r="H10" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+4)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="I10" s="45" t="str">
+      <x:c r="I10" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+4)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="J10" s="47" t="str">
+      <x:c r="J10" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+4)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="K10" s="49" t="str">
+      <x:c r="K10" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+4)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="L10" s="45" t="str">
+      <x:c r="L10" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+4)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="M10" s="47" t="str">
+      <x:c r="M10" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+4)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="N10" s="49" t="str">
+      <x:c r="N10" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+4)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+4))</x:f>
       </x:c>
-      <x:c r="O10" s="45" t="str">
+      <x:c r="O10" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+4)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+4))</x:f>
       </x:c>
       <x:c r="P10" s="14"/>
@@ -25820,7 +25915,7 @@
       <x:c r="D11" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+5)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+5))</x:f>
       </x:c>
-      <x:c r="E11" s="50" t="str">
+      <x:c r="E11" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+5)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+5))</x:f>
       </x:c>
       <x:c r="F11" s="23" t="str">
@@ -25829,7 +25924,7 @@
       <x:c r="G11" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+5)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+5))</x:f>
       </x:c>
-      <x:c r="H11" s="50" t="str">
+      <x:c r="H11" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+5)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+5))</x:f>
       </x:c>
       <x:c r="I11" s="23" t="str">
@@ -25838,7 +25933,7 @@
       <x:c r="J11" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+5)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+5))</x:f>
       </x:c>
-      <x:c r="K11" s="50" t="str">
+      <x:c r="K11" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+5)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+5))</x:f>
       </x:c>
       <x:c r="L11" s="23" t="str">
@@ -25847,7 +25942,7 @@
       <x:c r="M11" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+5)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+5))</x:f>
       </x:c>
-      <x:c r="N11" s="50" t="str">
+      <x:c r="N11" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+5)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+5))</x:f>
       </x:c>
       <x:c r="O11" s="23" t="str">
@@ -25860,43 +25955,43 @@
       <x:c r="B12" s="14" t="str">
         <x:v>历史分位</x:v>
       </x:c>
-      <x:c r="C12" s="45" t="str">
+      <x:c r="C12" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+6)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="D12" s="47" t="str">
+      <x:c r="D12" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+6)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="E12" s="49" t="str">
+      <x:c r="E12" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+6)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="F12" s="45" t="str">
+      <x:c r="F12" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+6)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="G12" s="47" t="str">
+      <x:c r="G12" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+6)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="H12" s="49" t="str">
+      <x:c r="H12" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+6)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="I12" s="45" t="str">
+      <x:c r="I12" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+6)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="J12" s="47" t="str">
+      <x:c r="J12" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+6)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="K12" s="49" t="str">
+      <x:c r="K12" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+6)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="L12" s="45" t="str">
+      <x:c r="L12" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+6)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="M12" s="47" t="str">
+      <x:c r="M12" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+6)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="N12" s="49" t="str">
+      <x:c r="N12" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+6)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+6))</x:f>
       </x:c>
-      <x:c r="O12" s="45" t="str">
+      <x:c r="O12" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+6)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+6))</x:f>
       </x:c>
       <x:c r="P12" s="14"/>
@@ -25912,7 +26007,7 @@
       <x:c r="D13" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+7)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+7))</x:f>
       </x:c>
-      <x:c r="E13" s="50" t="str">
+      <x:c r="E13" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+7)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+7))</x:f>
       </x:c>
       <x:c r="F13" s="23" t="str">
@@ -25921,7 +26016,7 @@
       <x:c r="G13" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+7)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+7))</x:f>
       </x:c>
-      <x:c r="H13" s="50" t="str">
+      <x:c r="H13" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+7)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+7))</x:f>
       </x:c>
       <x:c r="I13" s="23" t="str">
@@ -25930,7 +26025,7 @@
       <x:c r="J13" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+7)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+7))</x:f>
       </x:c>
-      <x:c r="K13" s="50" t="str">
+      <x:c r="K13" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+7)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+7))</x:f>
       </x:c>
       <x:c r="L13" s="23" t="str">
@@ -25939,7 +26034,7 @@
       <x:c r="M13" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+7)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+7))</x:f>
       </x:c>
-      <x:c r="N13" s="50" t="str">
+      <x:c r="N13" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+7)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+7))</x:f>
       </x:c>
       <x:c r="O13" s="23" t="str">
@@ -25952,43 +26047,43 @@
       <x:c r="B14" s="14" t="str">
         <x:v>短窗波动</x:v>
       </x:c>
-      <x:c r="C14" s="45" t="str">
+      <x:c r="C14" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+8)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="D14" s="47" t="str">
+      <x:c r="D14" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+8)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="E14" s="49" t="str">
+      <x:c r="E14" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+8)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="F14" s="45" t="str">
+      <x:c r="F14" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+8)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="G14" s="47" t="str">
+      <x:c r="G14" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+8)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="H14" s="49" t="str">
+      <x:c r="H14" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+8)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="I14" s="45" t="str">
+      <x:c r="I14" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+8)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="J14" s="47" t="str">
+      <x:c r="J14" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+8)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="K14" s="49" t="str">
+      <x:c r="K14" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+8)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="L14" s="45" t="str">
+      <x:c r="L14" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+8)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="M14" s="47" t="str">
+      <x:c r="M14" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+8)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="N14" s="49" t="str">
+      <x:c r="N14" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+8)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+8))</x:f>
       </x:c>
-      <x:c r="O14" s="45" t="str">
+      <x:c r="O14" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+8)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+8))</x:f>
       </x:c>
       <x:c r="P14" s="14"/>
@@ -26004,7 +26099,7 @@
       <x:c r="D15" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+9)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+9))</x:f>
       </x:c>
-      <x:c r="E15" s="50" t="str">
+      <x:c r="E15" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+9)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+9))</x:f>
       </x:c>
       <x:c r="F15" s="23" t="str">
@@ -26013,7 +26108,7 @@
       <x:c r="G15" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+9)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+9))</x:f>
       </x:c>
-      <x:c r="H15" s="50" t="str">
+      <x:c r="H15" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+9)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+9))</x:f>
       </x:c>
       <x:c r="I15" s="23" t="str">
@@ -26022,7 +26117,7 @@
       <x:c r="J15" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+9)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+9))</x:f>
       </x:c>
-      <x:c r="K15" s="50" t="str">
+      <x:c r="K15" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+9)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+9))</x:f>
       </x:c>
       <x:c r="L15" s="23" t="str">
@@ -26031,7 +26126,7 @@
       <x:c r="M15" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+9)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+9))</x:f>
       </x:c>
-      <x:c r="N15" s="50" t="str">
+      <x:c r="N15" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+9)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+9))</x:f>
       </x:c>
       <x:c r="O15" s="23" t="str">
@@ -26044,43 +26139,43 @@
       <x:c r="B16" s="14" t="str">
         <x:v>开盘缺口</x:v>
       </x:c>
-      <x:c r="C16" s="45" t="str">
+      <x:c r="C16" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+10)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="D16" s="47" t="str">
+      <x:c r="D16" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+10)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="E16" s="49" t="str">
+      <x:c r="E16" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+10)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="F16" s="45" t="str">
+      <x:c r="F16" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+10)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="G16" s="47" t="str">
+      <x:c r="G16" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+10)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="H16" s="49" t="str">
+      <x:c r="H16" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+10)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="I16" s="45" t="str">
+      <x:c r="I16" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+10)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="J16" s="47" t="str">
+      <x:c r="J16" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+10)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="K16" s="49" t="str">
+      <x:c r="K16" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+10)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="L16" s="45" t="str">
+      <x:c r="L16" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+10)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="M16" s="47" t="str">
+      <x:c r="M16" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+10)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="N16" s="49" t="str">
+      <x:c r="N16" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+10)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+10))</x:f>
       </x:c>
-      <x:c r="O16" s="45" t="str">
+      <x:c r="O16" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+10)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+10))</x:f>
       </x:c>
       <x:c r="P16" s="14"/>
@@ -26096,7 +26191,7 @@
       <x:c r="D17" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+11)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+11))</x:f>
       </x:c>
-      <x:c r="E17" s="50" t="str">
+      <x:c r="E17" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+11)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+11))</x:f>
       </x:c>
       <x:c r="F17" s="23" t="str">
@@ -26105,7 +26200,7 @@
       <x:c r="G17" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+11)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+11))</x:f>
       </x:c>
-      <x:c r="H17" s="50" t="str">
+      <x:c r="H17" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+11)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+11))</x:f>
       </x:c>
       <x:c r="I17" s="23" t="str">
@@ -26114,7 +26209,7 @@
       <x:c r="J17" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+11)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+11))</x:f>
       </x:c>
-      <x:c r="K17" s="50" t="str">
+      <x:c r="K17" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+11)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+11))</x:f>
       </x:c>
       <x:c r="L17" s="23" t="str">
@@ -26123,7 +26218,7 @@
       <x:c r="M17" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+11)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+11))</x:f>
       </x:c>
-      <x:c r="N17" s="50" t="str">
+      <x:c r="N17" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+11)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+11))</x:f>
       </x:c>
       <x:c r="O17" s="23" t="str">
@@ -26136,43 +26231,43 @@
       <x:c r="B18" s="14" t="str">
         <x:v>分钟中枢</x:v>
       </x:c>
-      <x:c r="C18" s="45" t="str">
+      <x:c r="C18" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+12)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="D18" s="47" t="str">
+      <x:c r="D18" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+12)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="E18" s="49" t="str">
+      <x:c r="E18" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+12)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="F18" s="45" t="str">
+      <x:c r="F18" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+12)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="G18" s="47" t="str">
+      <x:c r="G18" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+12)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="H18" s="49" t="str">
+      <x:c r="H18" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+12)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="I18" s="45" t="str">
+      <x:c r="I18" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+12)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="J18" s="47" t="str">
+      <x:c r="J18" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+12)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="K18" s="49" t="str">
+      <x:c r="K18" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+12)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="L18" s="45" t="str">
+      <x:c r="L18" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+12)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="M18" s="47" t="str">
+      <x:c r="M18" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+12)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="N18" s="49" t="str">
+      <x:c r="N18" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+12)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+12))</x:f>
       </x:c>
-      <x:c r="O18" s="45" t="str">
+      <x:c r="O18" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+12)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+12))</x:f>
       </x:c>
       <x:c r="P18" s="14"/>
@@ -26188,7 +26283,7 @@
       <x:c r="D19" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+13)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+13))</x:f>
       </x:c>
-      <x:c r="E19" s="50" t="str">
+      <x:c r="E19" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+13)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+13))</x:f>
       </x:c>
       <x:c r="F19" s="23" t="str">
@@ -26197,7 +26292,7 @@
       <x:c r="G19" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+13)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+13))</x:f>
       </x:c>
-      <x:c r="H19" s="50" t="str">
+      <x:c r="H19" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+13)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+13))</x:f>
       </x:c>
       <x:c r="I19" s="23" t="str">
@@ -26206,7 +26301,7 @@
       <x:c r="J19" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+13)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+13))</x:f>
       </x:c>
-      <x:c r="K19" s="50" t="str">
+      <x:c r="K19" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+13)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+13))</x:f>
       </x:c>
       <x:c r="L19" s="23" t="str">
@@ -26215,7 +26310,7 @@
       <x:c r="M19" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+13)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+13))</x:f>
       </x:c>
-      <x:c r="N19" s="50" t="str">
+      <x:c r="N19" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+13)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+13))</x:f>
       </x:c>
       <x:c r="O19" s="23" t="str">
@@ -26228,43 +26323,43 @@
       <x:c r="B20" s="14" t="str">
         <x:v>采集中枢</x:v>
       </x:c>
-      <x:c r="C20" s="45" t="str">
+      <x:c r="C20" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+14)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="D20" s="47" t="str">
+      <x:c r="D20" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+14)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="E20" s="49" t="str">
+      <x:c r="E20" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+14)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="F20" s="45" t="str">
+      <x:c r="F20" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+14)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="G20" s="47" t="str">
+      <x:c r="G20" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+14)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="H20" s="49" t="str">
+      <x:c r="H20" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+14)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="I20" s="45" t="str">
+      <x:c r="I20" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+14)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="J20" s="47" t="str">
+      <x:c r="J20" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+14)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="K20" s="49" t="str">
+      <x:c r="K20" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+14)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="L20" s="45" t="str">
+      <x:c r="L20" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+14)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="M20" s="47" t="str">
+      <x:c r="M20" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+14)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="N20" s="49" t="str">
+      <x:c r="N20" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+14)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+14))</x:f>
       </x:c>
-      <x:c r="O20" s="45" t="str">
+      <x:c r="O20" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+14)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+14))</x:f>
       </x:c>
       <x:c r="P20" s="14"/>
@@ -26280,7 +26375,7 @@
       <x:c r="D21" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+15)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+15))</x:f>
       </x:c>
-      <x:c r="E21" s="50" t="str">
+      <x:c r="E21" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+15)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+15))</x:f>
       </x:c>
       <x:c r="F21" s="23" t="str">
@@ -26289,7 +26384,7 @@
       <x:c r="G21" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+15)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+15))</x:f>
       </x:c>
-      <x:c r="H21" s="50" t="str">
+      <x:c r="H21" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+15)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+15))</x:f>
       </x:c>
       <x:c r="I21" s="23" t="str">
@@ -26298,7 +26393,7 @@
       <x:c r="J21" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+15)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+15))</x:f>
       </x:c>
-      <x:c r="K21" s="50" t="str">
+      <x:c r="K21" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+15)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+15))</x:f>
       </x:c>
       <x:c r="L21" s="23" t="str">
@@ -26307,7 +26402,7 @@
       <x:c r="M21" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+15)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+15))</x:f>
       </x:c>
-      <x:c r="N21" s="50" t="str">
+      <x:c r="N21" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+15)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+15))</x:f>
       </x:c>
       <x:c r="O21" s="23" t="str">
@@ -26320,43 +26415,43 @@
       <x:c r="B22" s="14" t="str">
         <x:v>增仓漂移</x:v>
       </x:c>
-      <x:c r="C22" s="45" t="str">
+      <x:c r="C22" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+16)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="D22" s="47" t="str">
+      <x:c r="D22" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+16)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="E22" s="49" t="str">
+      <x:c r="E22" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+16)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="F22" s="45" t="str">
+      <x:c r="F22" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+16)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="G22" s="47" t="str">
+      <x:c r="G22" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+16)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="H22" s="49" t="str">
+      <x:c r="H22" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+16)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="I22" s="45" t="str">
+      <x:c r="I22" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+16)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="J22" s="47" t="str">
+      <x:c r="J22" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+16)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="K22" s="49" t="str">
+      <x:c r="K22" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+16)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="L22" s="45" t="str">
+      <x:c r="L22" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+16)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="M22" s="47" t="str">
+      <x:c r="M22" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+16)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="N22" s="49" t="str">
+      <x:c r="N22" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+16)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+16))</x:f>
       </x:c>
-      <x:c r="O22" s="45" t="str">
+      <x:c r="O22" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+16)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+16))</x:f>
       </x:c>
       <x:c r="P22" s="14"/>
@@ -26372,7 +26467,7 @@
       <x:c r="D23" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+17)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+17))</x:f>
       </x:c>
-      <x:c r="E23" s="50" t="str">
+      <x:c r="E23" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+17)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+17))</x:f>
       </x:c>
       <x:c r="F23" s="23" t="str">
@@ -26381,7 +26476,7 @@
       <x:c r="G23" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+17)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+17))</x:f>
       </x:c>
-      <x:c r="H23" s="50" t="str">
+      <x:c r="H23" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+17)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+17))</x:f>
       </x:c>
       <x:c r="I23" s="23" t="str">
@@ -26390,7 +26485,7 @@
       <x:c r="J23" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+17)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+17))</x:f>
       </x:c>
-      <x:c r="K23" s="50" t="str">
+      <x:c r="K23" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+17)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+17))</x:f>
       </x:c>
       <x:c r="L23" s="23" t="str">
@@ -26399,7 +26494,7 @@
       <x:c r="M23" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+17)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+17))</x:f>
       </x:c>
-      <x:c r="N23" s="50" t="str">
+      <x:c r="N23" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+17)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+17))</x:f>
       </x:c>
       <x:c r="O23" s="23" t="str">
@@ -26412,43 +26507,43 @@
       <x:c r="B24" s="14" t="str">
         <x:v>增仓占比</x:v>
       </x:c>
-      <x:c r="C24" s="45" t="str">
+      <x:c r="C24" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+18)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="D24" s="47" t="str">
+      <x:c r="D24" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+18)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="E24" s="49" t="str">
+      <x:c r="E24" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+18)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="F24" s="45" t="str">
+      <x:c r="F24" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+18)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="G24" s="47" t="str">
+      <x:c r="G24" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+18)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="H24" s="49" t="str">
+      <x:c r="H24" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+18)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="I24" s="45" t="str">
+      <x:c r="I24" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+18)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="J24" s="47" t="str">
+      <x:c r="J24" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+18)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="K24" s="49" t="str">
+      <x:c r="K24" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+18)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="L24" s="45" t="str">
+      <x:c r="L24" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+18)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="M24" s="47" t="str">
+      <x:c r="M24" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+18)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="N24" s="49" t="str">
+      <x:c r="N24" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+18)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+18))</x:f>
       </x:c>
-      <x:c r="O24" s="45" t="str">
+      <x:c r="O24" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+18)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+18))</x:f>
       </x:c>
       <x:c r="P24" s="14"/>
@@ -26464,7 +26559,7 @@
       <x:c r="D25" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+19)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+19))</x:f>
       </x:c>
-      <x:c r="E25" s="50" t="str">
+      <x:c r="E25" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+19)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+19))</x:f>
       </x:c>
       <x:c r="F25" s="23" t="str">
@@ -26473,7 +26568,7 @@
       <x:c r="G25" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+19)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+19))</x:f>
       </x:c>
-      <x:c r="H25" s="50" t="str">
+      <x:c r="H25" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+19)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+19))</x:f>
       </x:c>
       <x:c r="I25" s="23" t="str">
@@ -26482,7 +26577,7 @@
       <x:c r="J25" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+19)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+19))</x:f>
       </x:c>
-      <x:c r="K25" s="50" t="str">
+      <x:c r="K25" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+19)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+19))</x:f>
       </x:c>
       <x:c r="L25" s="23" t="str">
@@ -26491,7 +26586,7 @@
       <x:c r="M25" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+19)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+19))</x:f>
       </x:c>
-      <x:c r="N25" s="50" t="str">
+      <x:c r="N25" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+19)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+19))</x:f>
       </x:c>
       <x:c r="O25" s="23" t="str">
@@ -26504,43 +26599,43 @@
       <x:c r="B26" s="14" t="str">
         <x:v>收盘位置差</x:v>
       </x:c>
-      <x:c r="C26" s="45" t="str">
+      <x:c r="C26" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+20)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="D26" s="47" t="str">
+      <x:c r="D26" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+20)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="E26" s="49" t="str">
+      <x:c r="E26" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+20)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="F26" s="45" t="str">
+      <x:c r="F26" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+20)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="G26" s="47" t="str">
+      <x:c r="G26" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+20)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="H26" s="49" t="str">
+      <x:c r="H26" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+20)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="I26" s="45" t="str">
+      <x:c r="I26" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+20)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="J26" s="47" t="str">
+      <x:c r="J26" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+20)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="K26" s="49" t="str">
+      <x:c r="K26" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+20)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="L26" s="45" t="str">
+      <x:c r="L26" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+20)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="M26" s="47" t="str">
+      <x:c r="M26" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+20)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="N26" s="49" t="str">
+      <x:c r="N26" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+20)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+20))</x:f>
       </x:c>
-      <x:c r="O26" s="45" t="str">
+      <x:c r="O26" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+20)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+20))</x:f>
       </x:c>
       <x:c r="P26" s="14"/>
@@ -26556,7 +26651,7 @@
       <x:c r="D27" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+21)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+21))</x:f>
       </x:c>
-      <x:c r="E27" s="50" t="str">
+      <x:c r="E27" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+21)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+21))</x:f>
       </x:c>
       <x:c r="F27" s="23" t="str">
@@ -26565,7 +26660,7 @@
       <x:c r="G27" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+21)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+21))</x:f>
       </x:c>
-      <x:c r="H27" s="50" t="str">
+      <x:c r="H27" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+21)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+21))</x:f>
       </x:c>
       <x:c r="I27" s="23" t="str">
@@ -26574,7 +26669,7 @@
       <x:c r="J27" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+21)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+21))</x:f>
       </x:c>
-      <x:c r="K27" s="50" t="str">
+      <x:c r="K27" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+21)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+21))</x:f>
       </x:c>
       <x:c r="L27" s="23" t="str">
@@ -26583,7 +26678,7 @@
       <x:c r="M27" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+21)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+21))</x:f>
       </x:c>
-      <x:c r="N27" s="50" t="str">
+      <x:c r="N27" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+21)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+21))</x:f>
       </x:c>
       <x:c r="O27" s="23" t="str">
@@ -26596,43 +26691,43 @@
       <x:c r="B28" s="14" t="str">
         <x:v>路径效率</x:v>
       </x:c>
-      <x:c r="C28" s="45" t="str">
+      <x:c r="C28" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+22)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="D28" s="47" t="str">
+      <x:c r="D28" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+22)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="E28" s="49" t="str">
+      <x:c r="E28" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+22)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="F28" s="45" t="str">
+      <x:c r="F28" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+22)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="G28" s="47" t="str">
+      <x:c r="G28" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+22)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="H28" s="49" t="str">
+      <x:c r="H28" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+22)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="I28" s="45" t="str">
+      <x:c r="I28" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+22)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="J28" s="47" t="str">
+      <x:c r="J28" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+22)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="K28" s="49" t="str">
+      <x:c r="K28" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+22)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="L28" s="45" t="str">
+      <x:c r="L28" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+22)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="M28" s="47" t="str">
+      <x:c r="M28" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+22)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="N28" s="49" t="str">
+      <x:c r="N28" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+22)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+22))</x:f>
       </x:c>
-      <x:c r="O28" s="45" t="str">
+      <x:c r="O28" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+22)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+22))</x:f>
       </x:c>
       <x:c r="P28" s="14"/>
@@ -26648,7 +26743,7 @@
       <x:c r="D29" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+23)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+23))</x:f>
       </x:c>
-      <x:c r="E29" s="50" t="str">
+      <x:c r="E29" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+23)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+23))</x:f>
       </x:c>
       <x:c r="F29" s="23" t="str">
@@ -26657,7 +26752,7 @@
       <x:c r="G29" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+23)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+23))</x:f>
       </x:c>
-      <x:c r="H29" s="50" t="str">
+      <x:c r="H29" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+23)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+23))</x:f>
       </x:c>
       <x:c r="I29" s="23" t="str">
@@ -26666,7 +26761,7 @@
       <x:c r="J29" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+23)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+23))</x:f>
       </x:c>
-      <x:c r="K29" s="50" t="str">
+      <x:c r="K29" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+23)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+23))</x:f>
       </x:c>
       <x:c r="L29" s="23" t="str">
@@ -26675,7 +26770,7 @@
       <x:c r="M29" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+23)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+23))</x:f>
       </x:c>
-      <x:c r="N29" s="50" t="str">
+      <x:c r="N29" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+23)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+23))</x:f>
       </x:c>
       <x:c r="O29" s="23" t="str">
@@ -26688,43 +26783,43 @@
       <x:c r="B30" s="14" t="str">
         <x:v>成本带</x:v>
       </x:c>
-      <x:c r="C30" s="45" t="str">
+      <x:c r="C30" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!D$7:D$406,$E$3*25+24)),"",INDEX('指标数据'!D$7:D$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="D30" s="47" t="str">
+      <x:c r="D30" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+24)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="E30" s="49" t="str">
+      <x:c r="E30" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+24)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="F30" s="45" t="str">
+      <x:c r="F30" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!G$7:G$406,$E$3*25+24)),"",INDEX('指标数据'!G$7:G$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="G30" s="47" t="str">
+      <x:c r="G30" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+24)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="H30" s="49" t="str">
+      <x:c r="H30" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+24)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="I30" s="45" t="str">
+      <x:c r="I30" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!J$7:J$406,$E$3*25+24)),"",INDEX('指标数据'!J$7:J$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="J30" s="47" t="str">
+      <x:c r="J30" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+24)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="K30" s="49" t="str">
+      <x:c r="K30" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+24)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="L30" s="45" t="str">
+      <x:c r="L30" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!M$7:M$406,$E$3*25+24)),"",INDEX('指标数据'!M$7:M$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="M30" s="47" t="str">
+      <x:c r="M30" s="48" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+24)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="N30" s="49" t="str">
+      <x:c r="N30" s="50" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+24)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+24))</x:f>
       </x:c>
-      <x:c r="O30" s="45" t="str">
+      <x:c r="O30" s="46" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!P$7:P$406,$E$3*25+24)),"",INDEX('指标数据'!P$7:P$406,$E$3*25+24))</x:f>
       </x:c>
       <x:c r="P30" s="14"/>
@@ -26740,7 +26835,7 @@
       <x:c r="D31" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!E$7:E$406,$E$3*25+25)),"",INDEX('指标数据'!E$7:E$406,$E$3*25+25))</x:f>
       </x:c>
-      <x:c r="E31" s="50" t="str">
+      <x:c r="E31" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!F$7:F$406,$E$3*25+25)),"",INDEX('指标数据'!F$7:F$406,$E$3*25+25))</x:f>
       </x:c>
       <x:c r="F31" s="23" t="str">
@@ -26749,7 +26844,7 @@
       <x:c r="G31" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!H$7:H$406,$E$3*25+25)),"",INDEX('指标数据'!H$7:H$406,$E$3*25+25))</x:f>
       </x:c>
-      <x:c r="H31" s="50" t="str">
+      <x:c r="H31" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!I$7:I$406,$E$3*25+25)),"",INDEX('指标数据'!I$7:I$406,$E$3*25+25))</x:f>
       </x:c>
       <x:c r="I31" s="23" t="str">
@@ -26758,7 +26853,7 @@
       <x:c r="J31" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!K$7:K$406,$E$3*25+25)),"",INDEX('指标数据'!K$7:K$406,$E$3*25+25))</x:f>
       </x:c>
-      <x:c r="K31" s="50" t="str">
+      <x:c r="K31" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!L$7:L$406,$E$3*25+25)),"",INDEX('指标数据'!L$7:L$406,$E$3*25+25))</x:f>
       </x:c>
       <x:c r="L31" s="23" t="str">
@@ -26767,7 +26862,7 @@
       <x:c r="M31" s="33" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!N$7:N$406,$E$3*25+25)),"",INDEX('指标数据'!N$7:N$406,$E$3*25+25))</x:f>
       </x:c>
-      <x:c r="N31" s="50" t="str">
+      <x:c r="N31" s="51" t="str">
         <x:f>IF(ISBLANK(INDEX('指标数据'!O$7:O$406,$E$3*25+25)),"",INDEX('指标数据'!O$7:O$406,$E$3*25+25))</x:f>
       </x:c>
       <x:c r="O31" s="23" t="str">
@@ -26813,92 +26908,92 @@
     </x:row>
     <x:row r="34" ht="19" customHeight="1">
       <x:c r="A34" s="14"/>
-      <x:c r="B34" s="41" t="str">
+      <x:c r="B34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="C34" s="41" t="str">
+      <x:c r="C34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="D34" s="41" t="str">
+      <x:c r="D34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="E34" s="41" t="str">
+      <x:c r="E34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="F34" s="41" t="str">
+      <x:c r="F34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="G34" s="41" t="str">
+      <x:c r="G34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="H34" s="41" t="str">
+      <x:c r="H34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="I34" s="41" t="str">
+      <x:c r="I34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="J34" s="41" t="str">
+      <x:c r="J34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="K34" s="41" t="str">
+      <x:c r="K34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="L34" s="41" t="str">
+      <x:c r="L34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="M34" s="41" t="str">
+      <x:c r="M34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="N34" s="41" t="str">
+      <x:c r="N34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
-      <x:c r="O34" s="41" t="str">
+      <x:c r="O34" s="42" t="str">
         <x:v>样本/分母：历史不足、输入缺失或分母无效；完整原因见研究指标。</x:v>
       </x:c>
       <x:c r="P34" s="14"/>
     </x:row>
     <x:row r="35" ht="19" customHeight="1">
       <x:c r="A35" s="14"/>
-      <x:c r="B35" s="41" t="str">
+      <x:c r="B35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="C35" s="41" t="str">
+      <x:c r="C35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="D35" s="41" t="str">
+      <x:c r="D35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="E35" s="41" t="str">
+      <x:c r="E35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="F35" s="41" t="str">
+      <x:c r="F35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="G35" s="41" t="str">
+      <x:c r="G35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="H35" s="41" t="str">
+      <x:c r="H35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="I35" s="41" t="str">
+      <x:c r="I35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="J35" s="41" t="str">
+      <x:c r="J35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="K35" s="41" t="str">
+      <x:c r="K35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="L35" s="41" t="str">
+      <x:c r="L35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="M35" s="41" t="str">
+      <x:c r="M35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="N35" s="41" t="str">
+      <x:c r="N35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
-      <x:c r="O35" s="41" t="str">
+      <x:c r="O35" s="42" t="str">
         <x:v>未连接 · 保存文件为快照</x:v>
       </x:c>
       <x:c r="P35" s="14"/>
@@ -26991,4 +27086,1905 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF087E8B"/>
+  </x:sheetPr>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="12" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="12" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" customHeight="1">
+      <x:c r="A1" s="53"/>
+      <x:c r="B1" s="53"/>
+      <x:c r="C1" s="53"/>
+      <x:c r="D1" s="53"/>
+      <x:c r="E1" s="53"/>
+      <x:c r="F1" s="53"/>
+      <x:c r="G1" s="53"/>
+      <x:c r="H1" s="53"/>
+      <x:c r="I1" s="53"/>
+      <x:c r="J1" s="53"/>
+      <x:c r="K1" s="53"/>
+      <x:c r="L1" s="53"/>
+      <x:c r="M1" s="53"/>
+      <x:c r="N1" s="53"/>
+      <x:c r="O1" s="53"/>
+      <x:c r="P1" s="53"/>
+    </x:row>
+    <x:row r="2" ht="24" customHeight="1">
+      <x:c r="A2" s="15" t="str">
+        <x:v>DELTA1  关注组合</x:v>
+      </x:c>
+      <x:c r="B2" s="53"/>
+      <x:c r="C2" s="53"/>
+      <x:c r="D2" s="53"/>
+      <x:c r="E2" s="53"/>
+      <x:c r="F2" s="53"/>
+      <x:c r="G2" s="53"/>
+      <x:c r="H2" s="53"/>
+      <x:c r="I2" s="53"/>
+      <x:c r="J2" s="53"/>
+      <x:c r="K2" s="53"/>
+      <x:c r="L2" s="53"/>
+      <x:c r="M2" s="53"/>
+      <x:c r="N2" s="53"/>
+      <x:c r="O2" s="53"/>
+      <x:c r="P2" s="53"/>
+    </x:row>
+    <x:row r="3" ht="24" customHeight="1">
+      <x:c r="A3" s="53" t="str">
+        <x:v>指标分类</x:v>
+      </x:c>
+      <x:c r="B3" s="56" t="str">
+        <x:v>全部</x:v>
+      </x:c>
+      <x:c r="C3" s="53"/>
+      <x:c r="D3" s="53" t="str">
+        <x:v>研究第几组</x:v>
+      </x:c>
+      <x:c r="E3" s="56" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F3" s="53"/>
+      <x:c r="G3" s="53"/>
+      <x:c r="H3" s="53"/>
+      <x:c r="I3" s="53"/>
+      <x:c r="J3" s="53"/>
+      <x:c r="K3" s="53"/>
+      <x:c r="L3" s="53"/>
+      <x:c r="M3" s="53"/>
+      <x:c r="N3" s="53"/>
+      <x:c r="O3" s="53"/>
+      <x:c r="P3" s="53"/>
+    </x:row>
+    <x:row r="4" ht="24" customHeight="1">
+      <x:c r="A4" s="54" t="str">
+        <x:v>黄色格可选；期现B留空自动配指数。历史日期填YYYY-MM-DD。组合保存在本机。</x:v>
+      </x:c>
+      <x:c r="B4" s="53"/>
+      <x:c r="C4" s="53"/>
+      <x:c r="D4" s="53"/>
+      <x:c r="E4" s="53"/>
+      <x:c r="F4" s="53"/>
+      <x:c r="G4" s="53"/>
+      <x:c r="H4" s="53"/>
+      <x:c r="I4" s="53"/>
+      <x:c r="J4" s="53"/>
+      <x:c r="K4" s="53"/>
+      <x:c r="L4" s="53"/>
+      <x:c r="M4" s="53"/>
+      <x:c r="N4" s="53"/>
+      <x:c r="O4" s="53"/>
+      <x:c r="P4" s="53"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="55" t="str">
+        <x:v>未连接 · 仅启动器维护的窗口可计算选择</x:v>
+      </x:c>
+      <x:c r="B5" s="53"/>
+      <x:c r="C5" s="53"/>
+      <x:c r="D5" s="53"/>
+      <x:c r="E5" s="53"/>
+      <x:c r="F5" s="53"/>
+      <x:c r="G5" s="53"/>
+      <x:c r="H5" s="53"/>
+      <x:c r="I5" s="53"/>
+      <x:c r="J5" s="53"/>
+      <x:c r="K5" s="53"/>
+      <x:c r="L5" s="53"/>
+      <x:c r="M5" s="53"/>
+      <x:c r="N5" s="53"/>
+      <x:c r="O5" s="53"/>
+      <x:c r="P5" s="53"/>
+    </x:row>
+    <x:row r="6" ht="28" customHeight="1">
+      <x:c r="A6" s="65" t="str">
+        <x:v>类型</x:v>
+      </x:c>
+      <x:c r="B6" s="65" t="str">
+        <x:v>合约A</x:v>
+      </x:c>
+      <x:c r="C6" s="65" t="str">
+        <x:v>合约B / 指数</x:v>
+      </x:c>
+      <x:c r="D6" s="65" t="str">
+        <x:v>输入</x:v>
+      </x:c>
+      <x:c r="E6" s="65" t="str">
+        <x:v>时点</x:v>
+      </x:c>
+      <x:c r="F6" s="65" t="str">
+        <x:v>历史日期</x:v>
+      </x:c>
+      <x:c r="G6" s="65" t="str">
+        <x:v>输入值</x:v>
+      </x:c>
+      <x:c r="H6" s="65" t="str">
+        <x:v>单位</x:v>
+      </x:c>
+      <x:c r="I6" s="65" t="str">
+        <x:v>路径效率</x:v>
+      </x:c>
+      <x:c r="J6" s="65" t="str">
+        <x:v>Z</x:v>
+      </x:c>
+      <x:c r="K6" s="65" t="str">
+        <x:v>A腿日内换手</x:v>
+      </x:c>
+      <x:c r="L6" s="65" t="str">
+        <x:v>同刻活跃</x:v>
+      </x:c>
+      <x:c r="M6" s="65" t="str">
+        <x:v>振幅</x:v>
+      </x:c>
+      <x:c r="N6" s="65" t="str">
+        <x:v>盘中源时</x:v>
+      </x:c>
+      <x:c r="O6" s="65" t="str">
+        <x:v>日终日期</x:v>
+      </x:c>
+      <x:c r="P6" s="65" t="str">
+        <x:v>状态</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="24" customHeight="1">
+      <x:c r="A7" s="56"/>
+      <x:c r="B7" s="56"/>
+      <x:c r="C7" s="56"/>
+      <x:c r="D7" s="56"/>
+      <x:c r="E7" s="56"/>
+      <x:c r="F7" s="57"/>
+      <x:c r="G7" s="58"/>
+      <x:c r="H7" s="58"/>
+      <x:c r="I7" s="58"/>
+      <x:c r="J7" s="58"/>
+      <x:c r="K7" s="58"/>
+      <x:c r="L7" s="58"/>
+      <x:c r="M7" s="58"/>
+      <x:c r="N7" s="59"/>
+      <x:c r="O7" s="60"/>
+      <x:c r="P7" s="53"/>
+    </x:row>
+    <x:row r="8" ht="24" customHeight="1">
+      <x:c r="A8" s="56"/>
+      <x:c r="B8" s="56"/>
+      <x:c r="C8" s="56"/>
+      <x:c r="D8" s="56"/>
+      <x:c r="E8" s="56"/>
+      <x:c r="F8" s="57"/>
+      <x:c r="G8" s="58"/>
+      <x:c r="H8" s="58"/>
+      <x:c r="I8" s="58"/>
+      <x:c r="J8" s="58"/>
+      <x:c r="K8" s="58"/>
+      <x:c r="L8" s="58"/>
+      <x:c r="M8" s="58"/>
+      <x:c r="N8" s="59"/>
+      <x:c r="O8" s="60"/>
+      <x:c r="P8" s="53"/>
+    </x:row>
+    <x:row r="9" ht="24" customHeight="1">
+      <x:c r="A9" s="56"/>
+      <x:c r="B9" s="56"/>
+      <x:c r="C9" s="56"/>
+      <x:c r="D9" s="56"/>
+      <x:c r="E9" s="56"/>
+      <x:c r="F9" s="57"/>
+      <x:c r="G9" s="58"/>
+      <x:c r="H9" s="58"/>
+      <x:c r="I9" s="58"/>
+      <x:c r="J9" s="58"/>
+      <x:c r="K9" s="58"/>
+      <x:c r="L9" s="58"/>
+      <x:c r="M9" s="58"/>
+      <x:c r="N9" s="59"/>
+      <x:c r="O9" s="60"/>
+      <x:c r="P9" s="53"/>
+    </x:row>
+    <x:row r="10" ht="24" customHeight="1">
+      <x:c r="A10" s="56"/>
+      <x:c r="B10" s="56"/>
+      <x:c r="C10" s="56"/>
+      <x:c r="D10" s="56"/>
+      <x:c r="E10" s="56"/>
+      <x:c r="F10" s="57"/>
+      <x:c r="G10" s="58"/>
+      <x:c r="H10" s="58"/>
+      <x:c r="I10" s="58"/>
+      <x:c r="J10" s="58"/>
+      <x:c r="K10" s="58"/>
+      <x:c r="L10" s="58"/>
+      <x:c r="M10" s="58"/>
+      <x:c r="N10" s="59"/>
+      <x:c r="O10" s="60"/>
+      <x:c r="P10" s="53"/>
+    </x:row>
+    <x:row r="11" ht="24" customHeight="1">
+      <x:c r="A11" s="56"/>
+      <x:c r="B11" s="56"/>
+      <x:c r="C11" s="56"/>
+      <x:c r="D11" s="56"/>
+      <x:c r="E11" s="56"/>
+      <x:c r="F11" s="57"/>
+      <x:c r="G11" s="58"/>
+      <x:c r="H11" s="58"/>
+      <x:c r="I11" s="58"/>
+      <x:c r="J11" s="58"/>
+      <x:c r="K11" s="58"/>
+      <x:c r="L11" s="58"/>
+      <x:c r="M11" s="58"/>
+      <x:c r="N11" s="59"/>
+      <x:c r="O11" s="60"/>
+      <x:c r="P11" s="53"/>
+    </x:row>
+    <x:row r="12" ht="24" customHeight="1">
+      <x:c r="A12" s="56"/>
+      <x:c r="B12" s="56"/>
+      <x:c r="C12" s="56"/>
+      <x:c r="D12" s="56"/>
+      <x:c r="E12" s="56"/>
+      <x:c r="F12" s="57"/>
+      <x:c r="G12" s="58"/>
+      <x:c r="H12" s="58"/>
+      <x:c r="I12" s="58"/>
+      <x:c r="J12" s="58"/>
+      <x:c r="K12" s="58"/>
+      <x:c r="L12" s="58"/>
+      <x:c r="M12" s="58"/>
+      <x:c r="N12" s="59"/>
+      <x:c r="O12" s="60"/>
+      <x:c r="P12" s="53"/>
+    </x:row>
+    <x:row r="13" ht="24" customHeight="1">
+      <x:c r="A13" s="56"/>
+      <x:c r="B13" s="56"/>
+      <x:c r="C13" s="56"/>
+      <x:c r="D13" s="56"/>
+      <x:c r="E13" s="56"/>
+      <x:c r="F13" s="57"/>
+      <x:c r="G13" s="58"/>
+      <x:c r="H13" s="58"/>
+      <x:c r="I13" s="58"/>
+      <x:c r="J13" s="58"/>
+      <x:c r="K13" s="58"/>
+      <x:c r="L13" s="58"/>
+      <x:c r="M13" s="58"/>
+      <x:c r="N13" s="59"/>
+      <x:c r="O13" s="60"/>
+      <x:c r="P13" s="53"/>
+    </x:row>
+    <x:row r="14" ht="24" customHeight="1">
+      <x:c r="A14" s="56"/>
+      <x:c r="B14" s="56"/>
+      <x:c r="C14" s="56"/>
+      <x:c r="D14" s="56"/>
+      <x:c r="E14" s="56"/>
+      <x:c r="F14" s="57"/>
+      <x:c r="G14" s="58"/>
+      <x:c r="H14" s="58"/>
+      <x:c r="I14" s="58"/>
+      <x:c r="J14" s="58"/>
+      <x:c r="K14" s="58"/>
+      <x:c r="L14" s="58"/>
+      <x:c r="M14" s="58"/>
+      <x:c r="N14" s="59"/>
+      <x:c r="O14" s="60"/>
+      <x:c r="P14" s="53"/>
+    </x:row>
+    <x:row r="15" ht="24" customHeight="1">
+      <x:c r="A15" s="53"/>
+      <x:c r="B15" s="53"/>
+      <x:c r="C15" s="53"/>
+      <x:c r="D15" s="53"/>
+      <x:c r="E15" s="53"/>
+      <x:c r="F15" s="53"/>
+      <x:c r="G15" s="53"/>
+      <x:c r="H15" s="53"/>
+      <x:c r="I15" s="53"/>
+      <x:c r="J15" s="53"/>
+      <x:c r="K15" s="53"/>
+      <x:c r="L15" s="53"/>
+      <x:c r="M15" s="53"/>
+      <x:c r="N15" s="53"/>
+      <x:c r="O15" s="53"/>
+      <x:c r="P15" s="53"/>
+    </x:row>
+    <x:row r="16" ht="24" customHeight="1">
+      <x:c r="A16" s="53"/>
+      <x:c r="B16" s="53"/>
+      <x:c r="C16" s="53"/>
+      <x:c r="D16" s="53"/>
+      <x:c r="E16" s="53"/>
+      <x:c r="F16" s="53"/>
+      <x:c r="G16" s="53"/>
+      <x:c r="H16" s="53"/>
+      <x:c r="I16" s="53"/>
+      <x:c r="J16" s="53"/>
+      <x:c r="K16" s="53"/>
+      <x:c r="L16" s="53"/>
+      <x:c r="M16" s="53"/>
+      <x:c r="N16" s="53"/>
+      <x:c r="O16" s="53"/>
+      <x:c r="P16" s="53"/>
+    </x:row>
+    <x:row r="17" ht="24" customHeight="1">
+      <x:c r="A17" s="61" t="str">
+        <x:v>选择上方组合，下面按分类列示盘中与日终结果</x:v>
+      </x:c>
+      <x:c r="B17" s="53"/>
+      <x:c r="C17" s="53"/>
+      <x:c r="D17" s="53"/>
+      <x:c r="E17" s="53"/>
+      <x:c r="F17" s="53"/>
+      <x:c r="G17" s="53"/>
+      <x:c r="H17" s="53"/>
+      <x:c r="I17" s="53"/>
+      <x:c r="J17" s="53"/>
+      <x:c r="K17" s="53"/>
+      <x:c r="L17" s="53"/>
+      <x:c r="M17" s="53"/>
+      <x:c r="N17" s="53"/>
+      <x:c r="O17" s="53"/>
+      <x:c r="P17" s="53"/>
+    </x:row>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="53"/>
+      <x:c r="B18" s="53"/>
+      <x:c r="C18" s="53"/>
+      <x:c r="D18" s="53"/>
+      <x:c r="E18" s="53"/>
+      <x:c r="F18" s="53"/>
+      <x:c r="G18" s="53"/>
+      <x:c r="H18" s="53"/>
+      <x:c r="I18" s="53"/>
+      <x:c r="J18" s="53"/>
+      <x:c r="K18" s="53"/>
+      <x:c r="L18" s="53"/>
+      <x:c r="M18" s="53"/>
+      <x:c r="N18" s="53"/>
+      <x:c r="O18" s="53"/>
+      <x:c r="P18" s="53"/>
+    </x:row>
+    <x:row r="19" ht="28" customHeight="1">
+      <x:c r="A19" s="65" t="str">
+        <x:v>分类</x:v>
+      </x:c>
+      <x:c r="B19" s="65" t="str">
+        <x:v>指标</x:v>
+      </x:c>
+      <x:c r="C19" s="65" t="str">
+        <x:v>单位</x:v>
+      </x:c>
+      <x:c r="D19" s="65" t="str">
+        <x:v>盘中值</x:v>
+      </x:c>
+      <x:c r="E19" s="65" t="str">
+        <x:v>盘中源时</x:v>
+      </x:c>
+      <x:c r="F19" s="65" t="str">
+        <x:v>盘中口径</x:v>
+      </x:c>
+      <x:c r="G19" s="65" t="str">
+        <x:v>日终值</x:v>
+      </x:c>
+      <x:c r="H19" s="65" t="str">
+        <x:v>日终日期</x:v>
+      </x:c>
+      <x:c r="I19" s="65" t="str">
+        <x:v>说明</x:v>
+      </x:c>
+      <x:c r="J19" s="53"/>
+      <x:c r="K19" s="53"/>
+      <x:c r="L19" s="53"/>
+      <x:c r="M19" s="53"/>
+      <x:c r="N19" s="53"/>
+      <x:c r="O19" s="53"/>
+      <x:c r="P19" s="53"/>
+    </x:row>
+    <x:row r="20" ht="38" customHeight="1">
+      <x:c r="A20" s="66"/>
+      <x:c r="B20" s="67"/>
+      <x:c r="C20" s="66"/>
+      <x:c r="D20" s="68"/>
+      <x:c r="E20" s="69"/>
+      <x:c r="F20" s="66"/>
+      <x:c r="G20" s="68"/>
+      <x:c r="H20" s="70"/>
+      <x:c r="I20" s="71"/>
+      <x:c r="J20" s="63"/>
+      <x:c r="K20" s="63"/>
+      <x:c r="L20" s="63"/>
+      <x:c r="M20" s="63"/>
+      <x:c r="N20" s="63"/>
+      <x:c r="O20" s="63"/>
+      <x:c r="P20" s="63"/>
+    </x:row>
+    <x:row r="21" ht="38" customHeight="1">
+      <x:c r="A21" s="53"/>
+      <x:c r="B21" s="62"/>
+      <x:c r="C21" s="53"/>
+      <x:c r="D21" s="58"/>
+      <x:c r="E21" s="59"/>
+      <x:c r="F21" s="53"/>
+      <x:c r="G21" s="58"/>
+      <x:c r="H21" s="60"/>
+      <x:c r="I21" s="63"/>
+      <x:c r="J21" s="63"/>
+      <x:c r="K21" s="63"/>
+      <x:c r="L21" s="63"/>
+      <x:c r="M21" s="63"/>
+      <x:c r="N21" s="63"/>
+      <x:c r="O21" s="63"/>
+      <x:c r="P21" s="63"/>
+    </x:row>
+    <x:row r="22" ht="38" customHeight="1">
+      <x:c r="A22" s="66"/>
+      <x:c r="B22" s="67"/>
+      <x:c r="C22" s="66"/>
+      <x:c r="D22" s="68"/>
+      <x:c r="E22" s="69"/>
+      <x:c r="F22" s="66"/>
+      <x:c r="G22" s="68"/>
+      <x:c r="H22" s="70"/>
+      <x:c r="I22" s="71"/>
+      <x:c r="J22" s="63"/>
+      <x:c r="K22" s="63"/>
+      <x:c r="L22" s="63"/>
+      <x:c r="M22" s="63"/>
+      <x:c r="N22" s="63"/>
+      <x:c r="O22" s="63"/>
+      <x:c r="P22" s="63"/>
+    </x:row>
+    <x:row r="23" ht="38" customHeight="1">
+      <x:c r="A23" s="53"/>
+      <x:c r="B23" s="62"/>
+      <x:c r="C23" s="53"/>
+      <x:c r="D23" s="58"/>
+      <x:c r="E23" s="59"/>
+      <x:c r="F23" s="53"/>
+      <x:c r="G23" s="58"/>
+      <x:c r="H23" s="60"/>
+      <x:c r="I23" s="63"/>
+      <x:c r="J23" s="63"/>
+      <x:c r="K23" s="63"/>
+      <x:c r="L23" s="63"/>
+      <x:c r="M23" s="63"/>
+      <x:c r="N23" s="63"/>
+      <x:c r="O23" s="63"/>
+      <x:c r="P23" s="63"/>
+    </x:row>
+    <x:row r="24" ht="38" customHeight="1">
+      <x:c r="A24" s="66"/>
+      <x:c r="B24" s="67"/>
+      <x:c r="C24" s="66"/>
+      <x:c r="D24" s="68"/>
+      <x:c r="E24" s="69"/>
+      <x:c r="F24" s="66"/>
+      <x:c r="G24" s="68"/>
+      <x:c r="H24" s="70"/>
+      <x:c r="I24" s="71"/>
+      <x:c r="J24" s="63"/>
+      <x:c r="K24" s="63"/>
+      <x:c r="L24" s="63"/>
+      <x:c r="M24" s="63"/>
+      <x:c r="N24" s="63"/>
+      <x:c r="O24" s="63"/>
+      <x:c r="P24" s="63"/>
+    </x:row>
+    <x:row r="25" ht="38" customHeight="1">
+      <x:c r="A25" s="53"/>
+      <x:c r="B25" s="62"/>
+      <x:c r="C25" s="53"/>
+      <x:c r="D25" s="58"/>
+      <x:c r="E25" s="59"/>
+      <x:c r="F25" s="53"/>
+      <x:c r="G25" s="58"/>
+      <x:c r="H25" s="60"/>
+      <x:c r="I25" s="63"/>
+      <x:c r="J25" s="63"/>
+      <x:c r="K25" s="63"/>
+      <x:c r="L25" s="63"/>
+      <x:c r="M25" s="63"/>
+      <x:c r="N25" s="63"/>
+      <x:c r="O25" s="63"/>
+      <x:c r="P25" s="63"/>
+    </x:row>
+    <x:row r="26" ht="38" customHeight="1">
+      <x:c r="A26" s="66"/>
+      <x:c r="B26" s="67"/>
+      <x:c r="C26" s="66"/>
+      <x:c r="D26" s="68"/>
+      <x:c r="E26" s="69"/>
+      <x:c r="F26" s="66"/>
+      <x:c r="G26" s="68"/>
+      <x:c r="H26" s="70"/>
+      <x:c r="I26" s="71"/>
+      <x:c r="J26" s="63"/>
+      <x:c r="K26" s="63"/>
+      <x:c r="L26" s="63"/>
+      <x:c r="M26" s="63"/>
+      <x:c r="N26" s="63"/>
+      <x:c r="O26" s="63"/>
+      <x:c r="P26" s="63"/>
+    </x:row>
+    <x:row r="27" ht="38" customHeight="1">
+      <x:c r="A27" s="53"/>
+      <x:c r="B27" s="62"/>
+      <x:c r="C27" s="53"/>
+      <x:c r="D27" s="58"/>
+      <x:c r="E27" s="59"/>
+      <x:c r="F27" s="53"/>
+      <x:c r="G27" s="58"/>
+      <x:c r="H27" s="60"/>
+      <x:c r="I27" s="63"/>
+      <x:c r="J27" s="63"/>
+      <x:c r="K27" s="63"/>
+      <x:c r="L27" s="63"/>
+      <x:c r="M27" s="63"/>
+      <x:c r="N27" s="63"/>
+      <x:c r="O27" s="63"/>
+      <x:c r="P27" s="63"/>
+    </x:row>
+    <x:row r="28" ht="38" customHeight="1">
+      <x:c r="A28" s="66"/>
+      <x:c r="B28" s="67"/>
+      <x:c r="C28" s="66"/>
+      <x:c r="D28" s="68"/>
+      <x:c r="E28" s="69"/>
+      <x:c r="F28" s="66"/>
+      <x:c r="G28" s="68"/>
+      <x:c r="H28" s="70"/>
+      <x:c r="I28" s="71"/>
+      <x:c r="J28" s="63"/>
+      <x:c r="K28" s="63"/>
+      <x:c r="L28" s="63"/>
+      <x:c r="M28" s="63"/>
+      <x:c r="N28" s="63"/>
+      <x:c r="O28" s="63"/>
+      <x:c r="P28" s="63"/>
+    </x:row>
+    <x:row r="29" ht="38" customHeight="1">
+      <x:c r="A29" s="53"/>
+      <x:c r="B29" s="62"/>
+      <x:c r="C29" s="53"/>
+      <x:c r="D29" s="58"/>
+      <x:c r="E29" s="59"/>
+      <x:c r="F29" s="53"/>
+      <x:c r="G29" s="58"/>
+      <x:c r="H29" s="60"/>
+      <x:c r="I29" s="63"/>
+      <x:c r="J29" s="63"/>
+      <x:c r="K29" s="63"/>
+      <x:c r="L29" s="63"/>
+      <x:c r="M29" s="63"/>
+      <x:c r="N29" s="63"/>
+      <x:c r="O29" s="63"/>
+      <x:c r="P29" s="63"/>
+    </x:row>
+    <x:row r="30" ht="38" customHeight="1">
+      <x:c r="A30" s="66"/>
+      <x:c r="B30" s="67"/>
+      <x:c r="C30" s="66"/>
+      <x:c r="D30" s="68"/>
+      <x:c r="E30" s="69"/>
+      <x:c r="F30" s="66"/>
+      <x:c r="G30" s="68"/>
+      <x:c r="H30" s="70"/>
+      <x:c r="I30" s="71"/>
+      <x:c r="J30" s="63"/>
+      <x:c r="K30" s="63"/>
+      <x:c r="L30" s="63"/>
+      <x:c r="M30" s="63"/>
+      <x:c r="N30" s="63"/>
+      <x:c r="O30" s="63"/>
+      <x:c r="P30" s="63"/>
+    </x:row>
+    <x:row r="31" ht="38" customHeight="1">
+      <x:c r="A31" s="53"/>
+      <x:c r="B31" s="62"/>
+      <x:c r="C31" s="53"/>
+      <x:c r="D31" s="58"/>
+      <x:c r="E31" s="59"/>
+      <x:c r="F31" s="53"/>
+      <x:c r="G31" s="58"/>
+      <x:c r="H31" s="60"/>
+      <x:c r="I31" s="63"/>
+      <x:c r="J31" s="63"/>
+      <x:c r="K31" s="63"/>
+      <x:c r="L31" s="63"/>
+      <x:c r="M31" s="63"/>
+      <x:c r="N31" s="63"/>
+      <x:c r="O31" s="63"/>
+      <x:c r="P31" s="63"/>
+    </x:row>
+    <x:row r="32" ht="38" customHeight="1">
+      <x:c r="A32" s="66"/>
+      <x:c r="B32" s="67"/>
+      <x:c r="C32" s="66"/>
+      <x:c r="D32" s="68"/>
+      <x:c r="E32" s="69"/>
+      <x:c r="F32" s="66"/>
+      <x:c r="G32" s="68"/>
+      <x:c r="H32" s="70"/>
+      <x:c r="I32" s="71"/>
+      <x:c r="J32" s="63"/>
+      <x:c r="K32" s="63"/>
+      <x:c r="L32" s="63"/>
+      <x:c r="M32" s="63"/>
+      <x:c r="N32" s="63"/>
+      <x:c r="O32" s="63"/>
+      <x:c r="P32" s="63"/>
+    </x:row>
+    <x:row r="33" ht="38" customHeight="1">
+      <x:c r="A33" s="53"/>
+      <x:c r="B33" s="62"/>
+      <x:c r="C33" s="53"/>
+      <x:c r="D33" s="58"/>
+      <x:c r="E33" s="59"/>
+      <x:c r="F33" s="53"/>
+      <x:c r="G33" s="58"/>
+      <x:c r="H33" s="60"/>
+      <x:c r="I33" s="63"/>
+      <x:c r="J33" s="63"/>
+      <x:c r="K33" s="63"/>
+      <x:c r="L33" s="63"/>
+      <x:c r="M33" s="63"/>
+      <x:c r="N33" s="63"/>
+      <x:c r="O33" s="63"/>
+      <x:c r="P33" s="63"/>
+    </x:row>
+    <x:row r="34" ht="38" customHeight="1">
+      <x:c r="A34" s="66"/>
+      <x:c r="B34" s="67"/>
+      <x:c r="C34" s="66"/>
+      <x:c r="D34" s="68"/>
+      <x:c r="E34" s="69"/>
+      <x:c r="F34" s="66"/>
+      <x:c r="G34" s="68"/>
+      <x:c r="H34" s="70"/>
+      <x:c r="I34" s="71"/>
+      <x:c r="J34" s="63"/>
+      <x:c r="K34" s="63"/>
+      <x:c r="L34" s="63"/>
+      <x:c r="M34" s="63"/>
+      <x:c r="N34" s="63"/>
+      <x:c r="O34" s="63"/>
+      <x:c r="P34" s="63"/>
+    </x:row>
+    <x:row r="35" ht="38" customHeight="1">
+      <x:c r="A35" s="53"/>
+      <x:c r="B35" s="62"/>
+      <x:c r="C35" s="53"/>
+      <x:c r="D35" s="58"/>
+      <x:c r="E35" s="59"/>
+      <x:c r="F35" s="53"/>
+      <x:c r="G35" s="58"/>
+      <x:c r="H35" s="60"/>
+      <x:c r="I35" s="63"/>
+      <x:c r="J35" s="63"/>
+      <x:c r="K35" s="63"/>
+      <x:c r="L35" s="63"/>
+      <x:c r="M35" s="63"/>
+      <x:c r="N35" s="63"/>
+      <x:c r="O35" s="63"/>
+      <x:c r="P35" s="63"/>
+    </x:row>
+    <x:row r="36" ht="38" customHeight="1">
+      <x:c r="A36" s="66"/>
+      <x:c r="B36" s="67"/>
+      <x:c r="C36" s="66"/>
+      <x:c r="D36" s="68"/>
+      <x:c r="E36" s="69"/>
+      <x:c r="F36" s="66"/>
+      <x:c r="G36" s="68"/>
+      <x:c r="H36" s="70"/>
+      <x:c r="I36" s="71"/>
+      <x:c r="J36" s="63"/>
+      <x:c r="K36" s="63"/>
+      <x:c r="L36" s="63"/>
+      <x:c r="M36" s="63"/>
+      <x:c r="N36" s="63"/>
+      <x:c r="O36" s="63"/>
+      <x:c r="P36" s="63"/>
+    </x:row>
+    <x:row r="37" ht="38" customHeight="1">
+      <x:c r="A37" s="53"/>
+      <x:c r="B37" s="62"/>
+      <x:c r="C37" s="53"/>
+      <x:c r="D37" s="58"/>
+      <x:c r="E37" s="59"/>
+      <x:c r="F37" s="53"/>
+      <x:c r="G37" s="58"/>
+      <x:c r="H37" s="60"/>
+      <x:c r="I37" s="63"/>
+      <x:c r="J37" s="63"/>
+      <x:c r="K37" s="63"/>
+      <x:c r="L37" s="63"/>
+      <x:c r="M37" s="63"/>
+      <x:c r="N37" s="63"/>
+      <x:c r="O37" s="63"/>
+      <x:c r="P37" s="63"/>
+    </x:row>
+    <x:row r="38" ht="38" customHeight="1">
+      <x:c r="A38" s="66"/>
+      <x:c r="B38" s="67"/>
+      <x:c r="C38" s="66"/>
+      <x:c r="D38" s="68"/>
+      <x:c r="E38" s="69"/>
+      <x:c r="F38" s="66"/>
+      <x:c r="G38" s="68"/>
+      <x:c r="H38" s="70"/>
+      <x:c r="I38" s="71"/>
+      <x:c r="J38" s="63"/>
+      <x:c r="K38" s="63"/>
+      <x:c r="L38" s="63"/>
+      <x:c r="M38" s="63"/>
+      <x:c r="N38" s="63"/>
+      <x:c r="O38" s="63"/>
+      <x:c r="P38" s="63"/>
+    </x:row>
+    <x:row r="39" ht="38" customHeight="1">
+      <x:c r="A39" s="53"/>
+      <x:c r="B39" s="62"/>
+      <x:c r="C39" s="53"/>
+      <x:c r="D39" s="58"/>
+      <x:c r="E39" s="59"/>
+      <x:c r="F39" s="53"/>
+      <x:c r="G39" s="58"/>
+      <x:c r="H39" s="60"/>
+      <x:c r="I39" s="63"/>
+      <x:c r="J39" s="63"/>
+      <x:c r="K39" s="63"/>
+      <x:c r="L39" s="63"/>
+      <x:c r="M39" s="63"/>
+      <x:c r="N39" s="63"/>
+      <x:c r="O39" s="63"/>
+      <x:c r="P39" s="63"/>
+    </x:row>
+    <x:row r="40" ht="38" customHeight="1">
+      <x:c r="A40" s="66"/>
+      <x:c r="B40" s="67"/>
+      <x:c r="C40" s="66"/>
+      <x:c r="D40" s="68"/>
+      <x:c r="E40" s="69"/>
+      <x:c r="F40" s="66"/>
+      <x:c r="G40" s="68"/>
+      <x:c r="H40" s="70"/>
+      <x:c r="I40" s="71"/>
+      <x:c r="J40" s="63"/>
+      <x:c r="K40" s="63"/>
+      <x:c r="L40" s="63"/>
+      <x:c r="M40" s="63"/>
+      <x:c r="N40" s="63"/>
+      <x:c r="O40" s="63"/>
+      <x:c r="P40" s="63"/>
+    </x:row>
+    <x:row r="41" ht="38" customHeight="1">
+      <x:c r="A41" s="53"/>
+      <x:c r="B41" s="62"/>
+      <x:c r="C41" s="53"/>
+      <x:c r="D41" s="58"/>
+      <x:c r="E41" s="59"/>
+      <x:c r="F41" s="53"/>
+      <x:c r="G41" s="58"/>
+      <x:c r="H41" s="60"/>
+      <x:c r="I41" s="63"/>
+      <x:c r="J41" s="63"/>
+      <x:c r="K41" s="63"/>
+      <x:c r="L41" s="63"/>
+      <x:c r="M41" s="63"/>
+      <x:c r="N41" s="63"/>
+      <x:c r="O41" s="63"/>
+      <x:c r="P41" s="63"/>
+    </x:row>
+    <x:row r="42" ht="38" customHeight="1">
+      <x:c r="A42" s="66"/>
+      <x:c r="B42" s="67"/>
+      <x:c r="C42" s="66"/>
+      <x:c r="D42" s="68"/>
+      <x:c r="E42" s="69"/>
+      <x:c r="F42" s="66"/>
+      <x:c r="G42" s="68"/>
+      <x:c r="H42" s="70"/>
+      <x:c r="I42" s="71"/>
+      <x:c r="J42" s="63"/>
+      <x:c r="K42" s="63"/>
+      <x:c r="L42" s="63"/>
+      <x:c r="M42" s="63"/>
+      <x:c r="N42" s="63"/>
+      <x:c r="O42" s="63"/>
+      <x:c r="P42" s="63"/>
+    </x:row>
+    <x:row r="43" ht="38" customHeight="1">
+      <x:c r="A43" s="53"/>
+      <x:c r="B43" s="62"/>
+      <x:c r="C43" s="53"/>
+      <x:c r="D43" s="58"/>
+      <x:c r="E43" s="59"/>
+      <x:c r="F43" s="53"/>
+      <x:c r="G43" s="58"/>
+      <x:c r="H43" s="60"/>
+      <x:c r="I43" s="63"/>
+      <x:c r="J43" s="63"/>
+      <x:c r="K43" s="63"/>
+      <x:c r="L43" s="63"/>
+      <x:c r="M43" s="63"/>
+      <x:c r="N43" s="63"/>
+      <x:c r="O43" s="63"/>
+      <x:c r="P43" s="63"/>
+    </x:row>
+    <x:row r="44" ht="38" customHeight="1">
+      <x:c r="A44" s="66"/>
+      <x:c r="B44" s="67"/>
+      <x:c r="C44" s="66"/>
+      <x:c r="D44" s="68"/>
+      <x:c r="E44" s="69"/>
+      <x:c r="F44" s="66"/>
+      <x:c r="G44" s="68"/>
+      <x:c r="H44" s="70"/>
+      <x:c r="I44" s="71"/>
+      <x:c r="J44" s="63"/>
+      <x:c r="K44" s="63"/>
+      <x:c r="L44" s="63"/>
+      <x:c r="M44" s="63"/>
+      <x:c r="N44" s="63"/>
+      <x:c r="O44" s="63"/>
+      <x:c r="P44" s="63"/>
+    </x:row>
+    <x:row r="45" ht="38" customHeight="1">
+      <x:c r="A45" s="53"/>
+      <x:c r="B45" s="62"/>
+      <x:c r="C45" s="53"/>
+      <x:c r="D45" s="58"/>
+      <x:c r="E45" s="59"/>
+      <x:c r="F45" s="53"/>
+      <x:c r="G45" s="58"/>
+      <x:c r="H45" s="60"/>
+      <x:c r="I45" s="63"/>
+      <x:c r="J45" s="63"/>
+      <x:c r="K45" s="63"/>
+      <x:c r="L45" s="63"/>
+      <x:c r="M45" s="63"/>
+      <x:c r="N45" s="63"/>
+      <x:c r="O45" s="63"/>
+      <x:c r="P45" s="63"/>
+    </x:row>
+    <x:row r="46" ht="38" customHeight="1">
+      <x:c r="A46" s="66"/>
+      <x:c r="B46" s="67"/>
+      <x:c r="C46" s="66"/>
+      <x:c r="D46" s="68"/>
+      <x:c r="E46" s="69"/>
+      <x:c r="F46" s="66"/>
+      <x:c r="G46" s="68"/>
+      <x:c r="H46" s="70"/>
+      <x:c r="I46" s="71"/>
+      <x:c r="J46" s="63"/>
+      <x:c r="K46" s="63"/>
+      <x:c r="L46" s="63"/>
+      <x:c r="M46" s="63"/>
+      <x:c r="N46" s="63"/>
+      <x:c r="O46" s="63"/>
+      <x:c r="P46" s="63"/>
+    </x:row>
+    <x:row r="47" ht="38" customHeight="1">
+      <x:c r="A47" s="53"/>
+      <x:c r="B47" s="62"/>
+      <x:c r="C47" s="53"/>
+      <x:c r="D47" s="58"/>
+      <x:c r="E47" s="59"/>
+      <x:c r="F47" s="53"/>
+      <x:c r="G47" s="58"/>
+      <x:c r="H47" s="60"/>
+      <x:c r="I47" s="63"/>
+      <x:c r="J47" s="63"/>
+      <x:c r="K47" s="63"/>
+      <x:c r="L47" s="63"/>
+      <x:c r="M47" s="63"/>
+      <x:c r="N47" s="63"/>
+      <x:c r="O47" s="63"/>
+      <x:c r="P47" s="63"/>
+    </x:row>
+    <x:row r="48" ht="38" customHeight="1">
+      <x:c r="A48" s="66"/>
+      <x:c r="B48" s="67"/>
+      <x:c r="C48" s="66"/>
+      <x:c r="D48" s="68"/>
+      <x:c r="E48" s="69"/>
+      <x:c r="F48" s="66"/>
+      <x:c r="G48" s="68"/>
+      <x:c r="H48" s="70"/>
+      <x:c r="I48" s="71"/>
+      <x:c r="J48" s="63"/>
+      <x:c r="K48" s="63"/>
+      <x:c r="L48" s="63"/>
+      <x:c r="M48" s="63"/>
+      <x:c r="N48" s="63"/>
+      <x:c r="O48" s="63"/>
+      <x:c r="P48" s="63"/>
+    </x:row>
+    <x:row r="49" ht="38" customHeight="1">
+      <x:c r="A49" s="53"/>
+      <x:c r="B49" s="62"/>
+      <x:c r="C49" s="53"/>
+      <x:c r="D49" s="58"/>
+      <x:c r="E49" s="59"/>
+      <x:c r="F49" s="53"/>
+      <x:c r="G49" s="58"/>
+      <x:c r="H49" s="60"/>
+      <x:c r="I49" s="63"/>
+      <x:c r="J49" s="63"/>
+      <x:c r="K49" s="63"/>
+      <x:c r="L49" s="63"/>
+      <x:c r="M49" s="63"/>
+      <x:c r="N49" s="63"/>
+      <x:c r="O49" s="63"/>
+      <x:c r="P49" s="63"/>
+    </x:row>
+    <x:row r="50" ht="38" customHeight="1">
+      <x:c r="A50" s="66"/>
+      <x:c r="B50" s="67"/>
+      <x:c r="C50" s="66"/>
+      <x:c r="D50" s="68"/>
+      <x:c r="E50" s="69"/>
+      <x:c r="F50" s="66"/>
+      <x:c r="G50" s="68"/>
+      <x:c r="H50" s="70"/>
+      <x:c r="I50" s="71"/>
+      <x:c r="J50" s="63"/>
+      <x:c r="K50" s="63"/>
+      <x:c r="L50" s="63"/>
+      <x:c r="M50" s="63"/>
+      <x:c r="N50" s="63"/>
+      <x:c r="O50" s="63"/>
+      <x:c r="P50" s="63"/>
+    </x:row>
+    <x:row r="51" ht="38" customHeight="1">
+      <x:c r="A51" s="53"/>
+      <x:c r="B51" s="62"/>
+      <x:c r="C51" s="53"/>
+      <x:c r="D51" s="58"/>
+      <x:c r="E51" s="59"/>
+      <x:c r="F51" s="53"/>
+      <x:c r="G51" s="58"/>
+      <x:c r="H51" s="60"/>
+      <x:c r="I51" s="63"/>
+      <x:c r="J51" s="63"/>
+      <x:c r="K51" s="63"/>
+      <x:c r="L51" s="63"/>
+      <x:c r="M51" s="63"/>
+      <x:c r="N51" s="63"/>
+      <x:c r="O51" s="63"/>
+      <x:c r="P51" s="63"/>
+    </x:row>
+    <x:row r="52" ht="38" customHeight="1">
+      <x:c r="A52" s="66"/>
+      <x:c r="B52" s="67"/>
+      <x:c r="C52" s="66"/>
+      <x:c r="D52" s="68"/>
+      <x:c r="E52" s="69"/>
+      <x:c r="F52" s="66"/>
+      <x:c r="G52" s="68"/>
+      <x:c r="H52" s="70"/>
+      <x:c r="I52" s="71"/>
+      <x:c r="J52" s="63"/>
+      <x:c r="K52" s="63"/>
+      <x:c r="L52" s="63"/>
+      <x:c r="M52" s="63"/>
+      <x:c r="N52" s="63"/>
+      <x:c r="O52" s="63"/>
+      <x:c r="P52" s="63"/>
+    </x:row>
+    <x:row r="53" ht="38" customHeight="1">
+      <x:c r="A53" s="53"/>
+      <x:c r="B53" s="62"/>
+      <x:c r="C53" s="53"/>
+      <x:c r="D53" s="58"/>
+      <x:c r="E53" s="59"/>
+      <x:c r="F53" s="53"/>
+      <x:c r="G53" s="58"/>
+      <x:c r="H53" s="60"/>
+      <x:c r="I53" s="63"/>
+      <x:c r="J53" s="63"/>
+      <x:c r="K53" s="63"/>
+      <x:c r="L53" s="63"/>
+      <x:c r="M53" s="63"/>
+      <x:c r="N53" s="63"/>
+      <x:c r="O53" s="63"/>
+      <x:c r="P53" s="63"/>
+    </x:row>
+    <x:row r="54" ht="38" customHeight="1">
+      <x:c r="A54" s="66"/>
+      <x:c r="B54" s="67"/>
+      <x:c r="C54" s="66"/>
+      <x:c r="D54" s="68"/>
+      <x:c r="E54" s="69"/>
+      <x:c r="F54" s="66"/>
+      <x:c r="G54" s="68"/>
+      <x:c r="H54" s="70"/>
+      <x:c r="I54" s="71"/>
+      <x:c r="J54" s="63"/>
+      <x:c r="K54" s="63"/>
+      <x:c r="L54" s="63"/>
+      <x:c r="M54" s="63"/>
+      <x:c r="N54" s="63"/>
+      <x:c r="O54" s="63"/>
+      <x:c r="P54" s="63"/>
+    </x:row>
+    <x:row r="55" ht="38" customHeight="1">
+      <x:c r="A55" s="53"/>
+      <x:c r="B55" s="62"/>
+      <x:c r="C55" s="53"/>
+      <x:c r="D55" s="58"/>
+      <x:c r="E55" s="59"/>
+      <x:c r="F55" s="53"/>
+      <x:c r="G55" s="58"/>
+      <x:c r="H55" s="60"/>
+      <x:c r="I55" s="63"/>
+      <x:c r="J55" s="63"/>
+      <x:c r="K55" s="63"/>
+      <x:c r="L55" s="63"/>
+      <x:c r="M55" s="63"/>
+      <x:c r="N55" s="63"/>
+      <x:c r="O55" s="63"/>
+      <x:c r="P55" s="63"/>
+    </x:row>
+    <x:row r="56" ht="38" customHeight="1">
+      <x:c r="A56" s="66"/>
+      <x:c r="B56" s="67"/>
+      <x:c r="C56" s="66"/>
+      <x:c r="D56" s="68"/>
+      <x:c r="E56" s="69"/>
+      <x:c r="F56" s="66"/>
+      <x:c r="G56" s="68"/>
+      <x:c r="H56" s="70"/>
+      <x:c r="I56" s="71"/>
+      <x:c r="J56" s="63"/>
+      <x:c r="K56" s="63"/>
+      <x:c r="L56" s="63"/>
+      <x:c r="M56" s="63"/>
+      <x:c r="N56" s="63"/>
+      <x:c r="O56" s="63"/>
+      <x:c r="P56" s="63"/>
+    </x:row>
+    <x:row r="57" ht="38" customHeight="1">
+      <x:c r="A57" s="53"/>
+      <x:c r="B57" s="62"/>
+      <x:c r="C57" s="53"/>
+      <x:c r="D57" s="58"/>
+      <x:c r="E57" s="59"/>
+      <x:c r="F57" s="53"/>
+      <x:c r="G57" s="58"/>
+      <x:c r="H57" s="60"/>
+      <x:c r="I57" s="63"/>
+      <x:c r="J57" s="63"/>
+      <x:c r="K57" s="63"/>
+      <x:c r="L57" s="63"/>
+      <x:c r="M57" s="63"/>
+      <x:c r="N57" s="63"/>
+      <x:c r="O57" s="63"/>
+      <x:c r="P57" s="63"/>
+    </x:row>
+    <x:row r="58" ht="38" customHeight="1">
+      <x:c r="A58" s="66"/>
+      <x:c r="B58" s="67"/>
+      <x:c r="C58" s="66"/>
+      <x:c r="D58" s="68"/>
+      <x:c r="E58" s="69"/>
+      <x:c r="F58" s="66"/>
+      <x:c r="G58" s="68"/>
+      <x:c r="H58" s="70"/>
+      <x:c r="I58" s="71"/>
+      <x:c r="J58" s="63"/>
+      <x:c r="K58" s="63"/>
+      <x:c r="L58" s="63"/>
+      <x:c r="M58" s="63"/>
+      <x:c r="N58" s="63"/>
+      <x:c r="O58" s="63"/>
+      <x:c r="P58" s="63"/>
+    </x:row>
+    <x:row r="59" ht="38" customHeight="1">
+      <x:c r="A59" s="53"/>
+      <x:c r="B59" s="62"/>
+      <x:c r="C59" s="53"/>
+      <x:c r="D59" s="58"/>
+      <x:c r="E59" s="59"/>
+      <x:c r="F59" s="53"/>
+      <x:c r="G59" s="58"/>
+      <x:c r="H59" s="60"/>
+      <x:c r="I59" s="63"/>
+      <x:c r="J59" s="63"/>
+      <x:c r="K59" s="63"/>
+      <x:c r="L59" s="63"/>
+      <x:c r="M59" s="63"/>
+      <x:c r="N59" s="63"/>
+      <x:c r="O59" s="63"/>
+      <x:c r="P59" s="63"/>
+    </x:row>
+    <x:row r="60" ht="38" customHeight="1">
+      <x:c r="A60" s="66"/>
+      <x:c r="B60" s="67"/>
+      <x:c r="C60" s="66"/>
+      <x:c r="D60" s="68"/>
+      <x:c r="E60" s="69"/>
+      <x:c r="F60" s="66"/>
+      <x:c r="G60" s="68"/>
+      <x:c r="H60" s="70"/>
+      <x:c r="I60" s="71"/>
+      <x:c r="J60" s="63"/>
+      <x:c r="K60" s="63"/>
+      <x:c r="L60" s="63"/>
+      <x:c r="M60" s="63"/>
+      <x:c r="N60" s="63"/>
+      <x:c r="O60" s="63"/>
+      <x:c r="P60" s="63"/>
+    </x:row>
+    <x:row r="61" ht="38" customHeight="1">
+      <x:c r="A61" s="53"/>
+      <x:c r="B61" s="62"/>
+      <x:c r="C61" s="53"/>
+      <x:c r="D61" s="58"/>
+      <x:c r="E61" s="59"/>
+      <x:c r="F61" s="53"/>
+      <x:c r="G61" s="58"/>
+      <x:c r="H61" s="60"/>
+      <x:c r="I61" s="63"/>
+      <x:c r="J61" s="63"/>
+      <x:c r="K61" s="63"/>
+      <x:c r="L61" s="63"/>
+      <x:c r="M61" s="63"/>
+      <x:c r="N61" s="63"/>
+      <x:c r="O61" s="63"/>
+      <x:c r="P61" s="63"/>
+    </x:row>
+    <x:row r="62" ht="38" customHeight="1">
+      <x:c r="A62" s="66"/>
+      <x:c r="B62" s="67"/>
+      <x:c r="C62" s="66"/>
+      <x:c r="D62" s="68"/>
+      <x:c r="E62" s="69"/>
+      <x:c r="F62" s="66"/>
+      <x:c r="G62" s="68"/>
+      <x:c r="H62" s="70"/>
+      <x:c r="I62" s="71"/>
+      <x:c r="J62" s="63"/>
+      <x:c r="K62" s="63"/>
+      <x:c r="L62" s="63"/>
+      <x:c r="M62" s="63"/>
+      <x:c r="N62" s="63"/>
+      <x:c r="O62" s="63"/>
+      <x:c r="P62" s="63"/>
+    </x:row>
+    <x:row r="63" ht="38" customHeight="1">
+      <x:c r="A63" s="53"/>
+      <x:c r="B63" s="62"/>
+      <x:c r="C63" s="53"/>
+      <x:c r="D63" s="58"/>
+      <x:c r="E63" s="59"/>
+      <x:c r="F63" s="53"/>
+      <x:c r="G63" s="58"/>
+      <x:c r="H63" s="60"/>
+      <x:c r="I63" s="63"/>
+      <x:c r="J63" s="63"/>
+      <x:c r="K63" s="63"/>
+      <x:c r="L63" s="63"/>
+      <x:c r="M63" s="63"/>
+      <x:c r="N63" s="63"/>
+      <x:c r="O63" s="63"/>
+      <x:c r="P63" s="63"/>
+    </x:row>
+    <x:row r="64" ht="38" customHeight="1">
+      <x:c r="A64" s="66"/>
+      <x:c r="B64" s="67"/>
+      <x:c r="C64" s="66"/>
+      <x:c r="D64" s="68"/>
+      <x:c r="E64" s="69"/>
+      <x:c r="F64" s="66"/>
+      <x:c r="G64" s="68"/>
+      <x:c r="H64" s="70"/>
+      <x:c r="I64" s="71"/>
+      <x:c r="J64" s="63"/>
+      <x:c r="K64" s="63"/>
+      <x:c r="L64" s="63"/>
+      <x:c r="M64" s="63"/>
+      <x:c r="N64" s="63"/>
+      <x:c r="O64" s="63"/>
+      <x:c r="P64" s="63"/>
+    </x:row>
+    <x:row r="65" ht="38" customHeight="1">
+      <x:c r="A65" s="53"/>
+      <x:c r="B65" s="62"/>
+      <x:c r="C65" s="53"/>
+      <x:c r="D65" s="58"/>
+      <x:c r="E65" s="59"/>
+      <x:c r="F65" s="53"/>
+      <x:c r="G65" s="58"/>
+      <x:c r="H65" s="60"/>
+      <x:c r="I65" s="63"/>
+      <x:c r="J65" s="63"/>
+      <x:c r="K65" s="63"/>
+      <x:c r="L65" s="63"/>
+      <x:c r="M65" s="63"/>
+      <x:c r="N65" s="63"/>
+      <x:c r="O65" s="63"/>
+      <x:c r="P65" s="63"/>
+    </x:row>
+    <x:row r="66" ht="38" customHeight="1">
+      <x:c r="A66" s="66"/>
+      <x:c r="B66" s="67"/>
+      <x:c r="C66" s="66"/>
+      <x:c r="D66" s="68"/>
+      <x:c r="E66" s="69"/>
+      <x:c r="F66" s="66"/>
+      <x:c r="G66" s="68"/>
+      <x:c r="H66" s="70"/>
+      <x:c r="I66" s="71"/>
+      <x:c r="J66" s="63"/>
+      <x:c r="K66" s="63"/>
+      <x:c r="L66" s="63"/>
+      <x:c r="M66" s="63"/>
+      <x:c r="N66" s="63"/>
+      <x:c r="O66" s="63"/>
+      <x:c r="P66" s="63"/>
+    </x:row>
+    <x:row r="67" ht="38" customHeight="1">
+      <x:c r="A67" s="53"/>
+      <x:c r="B67" s="62"/>
+      <x:c r="C67" s="53"/>
+      <x:c r="D67" s="58"/>
+      <x:c r="E67" s="59"/>
+      <x:c r="F67" s="53"/>
+      <x:c r="G67" s="58"/>
+      <x:c r="H67" s="60"/>
+      <x:c r="I67" s="63"/>
+      <x:c r="J67" s="63"/>
+      <x:c r="K67" s="63"/>
+      <x:c r="L67" s="63"/>
+      <x:c r="M67" s="63"/>
+      <x:c r="N67" s="63"/>
+      <x:c r="O67" s="63"/>
+      <x:c r="P67" s="63"/>
+    </x:row>
+    <x:row r="68" ht="38" customHeight="1">
+      <x:c r="A68" s="66"/>
+      <x:c r="B68" s="67"/>
+      <x:c r="C68" s="66"/>
+      <x:c r="D68" s="68"/>
+      <x:c r="E68" s="69"/>
+      <x:c r="F68" s="66"/>
+      <x:c r="G68" s="68"/>
+      <x:c r="H68" s="70"/>
+      <x:c r="I68" s="71"/>
+      <x:c r="J68" s="63"/>
+      <x:c r="K68" s="63"/>
+      <x:c r="L68" s="63"/>
+      <x:c r="M68" s="63"/>
+      <x:c r="N68" s="63"/>
+      <x:c r="O68" s="63"/>
+      <x:c r="P68" s="63"/>
+    </x:row>
+    <x:row r="69" ht="38" customHeight="1">
+      <x:c r="A69" s="53"/>
+      <x:c r="B69" s="62"/>
+      <x:c r="C69" s="53"/>
+      <x:c r="D69" s="58"/>
+      <x:c r="E69" s="59"/>
+      <x:c r="F69" s="53"/>
+      <x:c r="G69" s="58"/>
+      <x:c r="H69" s="60"/>
+      <x:c r="I69" s="63"/>
+      <x:c r="J69" s="63"/>
+      <x:c r="K69" s="63"/>
+      <x:c r="L69" s="63"/>
+      <x:c r="M69" s="63"/>
+      <x:c r="N69" s="63"/>
+      <x:c r="O69" s="63"/>
+      <x:c r="P69" s="63"/>
+    </x:row>
+    <x:row r="70" ht="38" customHeight="1">
+      <x:c r="A70" s="66"/>
+      <x:c r="B70" s="67"/>
+      <x:c r="C70" s="66"/>
+      <x:c r="D70" s="68"/>
+      <x:c r="E70" s="69"/>
+      <x:c r="F70" s="66"/>
+      <x:c r="G70" s="68"/>
+      <x:c r="H70" s="70"/>
+      <x:c r="I70" s="71"/>
+      <x:c r="J70" s="63"/>
+      <x:c r="K70" s="63"/>
+      <x:c r="L70" s="63"/>
+      <x:c r="M70" s="63"/>
+      <x:c r="N70" s="63"/>
+      <x:c r="O70" s="63"/>
+      <x:c r="P70" s="63"/>
+    </x:row>
+    <x:row r="71" ht="38" customHeight="1">
+      <x:c r="A71" s="53"/>
+      <x:c r="B71" s="62"/>
+      <x:c r="C71" s="53"/>
+      <x:c r="D71" s="58"/>
+      <x:c r="E71" s="59"/>
+      <x:c r="F71" s="53"/>
+      <x:c r="G71" s="58"/>
+      <x:c r="H71" s="60"/>
+      <x:c r="I71" s="63"/>
+      <x:c r="J71" s="63"/>
+      <x:c r="K71" s="63"/>
+      <x:c r="L71" s="63"/>
+      <x:c r="M71" s="63"/>
+      <x:c r="N71" s="63"/>
+      <x:c r="O71" s="63"/>
+      <x:c r="P71" s="63"/>
+    </x:row>
+    <x:row r="72" ht="38" customHeight="1">
+      <x:c r="A72" s="66"/>
+      <x:c r="B72" s="67"/>
+      <x:c r="C72" s="66"/>
+      <x:c r="D72" s="68"/>
+      <x:c r="E72" s="69"/>
+      <x:c r="F72" s="66"/>
+      <x:c r="G72" s="68"/>
+      <x:c r="H72" s="70"/>
+      <x:c r="I72" s="71"/>
+      <x:c r="J72" s="63"/>
+      <x:c r="K72" s="63"/>
+      <x:c r="L72" s="63"/>
+      <x:c r="M72" s="63"/>
+      <x:c r="N72" s="63"/>
+      <x:c r="O72" s="63"/>
+      <x:c r="P72" s="63"/>
+    </x:row>
+    <x:row r="73" ht="38" customHeight="1">
+      <x:c r="A73" s="53"/>
+      <x:c r="B73" s="62"/>
+      <x:c r="C73" s="53"/>
+      <x:c r="D73" s="58"/>
+      <x:c r="E73" s="59"/>
+      <x:c r="F73" s="53"/>
+      <x:c r="G73" s="58"/>
+      <x:c r="H73" s="60"/>
+      <x:c r="I73" s="63"/>
+      <x:c r="J73" s="63"/>
+      <x:c r="K73" s="63"/>
+      <x:c r="L73" s="63"/>
+      <x:c r="M73" s="63"/>
+      <x:c r="N73" s="63"/>
+      <x:c r="O73" s="63"/>
+      <x:c r="P73" s="63"/>
+    </x:row>
+    <x:row r="74" ht="38" customHeight="1">
+      <x:c r="A74" s="66"/>
+      <x:c r="B74" s="67"/>
+      <x:c r="C74" s="66"/>
+      <x:c r="D74" s="68"/>
+      <x:c r="E74" s="69"/>
+      <x:c r="F74" s="66"/>
+      <x:c r="G74" s="68"/>
+      <x:c r="H74" s="70"/>
+      <x:c r="I74" s="71"/>
+      <x:c r="J74" s="63"/>
+      <x:c r="K74" s="63"/>
+      <x:c r="L74" s="63"/>
+      <x:c r="M74" s="63"/>
+      <x:c r="N74" s="63"/>
+      <x:c r="O74" s="63"/>
+      <x:c r="P74" s="63"/>
+    </x:row>
+    <x:row r="75" ht="38" customHeight="1">
+      <x:c r="A75" s="53"/>
+      <x:c r="B75" s="62"/>
+      <x:c r="C75" s="53"/>
+      <x:c r="D75" s="58"/>
+      <x:c r="E75" s="59"/>
+      <x:c r="F75" s="53"/>
+      <x:c r="G75" s="58"/>
+      <x:c r="H75" s="60"/>
+      <x:c r="I75" s="63"/>
+      <x:c r="J75" s="63"/>
+      <x:c r="K75" s="63"/>
+      <x:c r="L75" s="63"/>
+      <x:c r="M75" s="63"/>
+      <x:c r="N75" s="63"/>
+      <x:c r="O75" s="63"/>
+      <x:c r="P75" s="63"/>
+    </x:row>
+    <x:row r="76" ht="38" customHeight="1">
+      <x:c r="A76" s="66"/>
+      <x:c r="B76" s="67"/>
+      <x:c r="C76" s="66"/>
+      <x:c r="D76" s="68"/>
+      <x:c r="E76" s="69"/>
+      <x:c r="F76" s="66"/>
+      <x:c r="G76" s="68"/>
+      <x:c r="H76" s="70"/>
+      <x:c r="I76" s="71"/>
+      <x:c r="J76" s="63"/>
+      <x:c r="K76" s="63"/>
+      <x:c r="L76" s="63"/>
+      <x:c r="M76" s="63"/>
+      <x:c r="N76" s="63"/>
+      <x:c r="O76" s="63"/>
+      <x:c r="P76" s="63"/>
+    </x:row>
+    <x:row r="77" ht="38" customHeight="1">
+      <x:c r="A77" s="53"/>
+      <x:c r="B77" s="62"/>
+      <x:c r="C77" s="53"/>
+      <x:c r="D77" s="58"/>
+      <x:c r="E77" s="59"/>
+      <x:c r="F77" s="53"/>
+      <x:c r="G77" s="58"/>
+      <x:c r="H77" s="60"/>
+      <x:c r="I77" s="63"/>
+      <x:c r="J77" s="63"/>
+      <x:c r="K77" s="63"/>
+      <x:c r="L77" s="63"/>
+      <x:c r="M77" s="63"/>
+      <x:c r="N77" s="63"/>
+      <x:c r="O77" s="63"/>
+      <x:c r="P77" s="63"/>
+    </x:row>
+    <x:row r="78" ht="38" customHeight="1">
+      <x:c r="A78" s="66"/>
+      <x:c r="B78" s="67"/>
+      <x:c r="C78" s="66"/>
+      <x:c r="D78" s="68"/>
+      <x:c r="E78" s="69"/>
+      <x:c r="F78" s="66"/>
+      <x:c r="G78" s="68"/>
+      <x:c r="H78" s="70"/>
+      <x:c r="I78" s="71"/>
+      <x:c r="J78" s="63"/>
+      <x:c r="K78" s="63"/>
+      <x:c r="L78" s="63"/>
+      <x:c r="M78" s="63"/>
+      <x:c r="N78" s="63"/>
+      <x:c r="O78" s="63"/>
+      <x:c r="P78" s="63"/>
+    </x:row>
+    <x:row r="79" ht="38" customHeight="1">
+      <x:c r="A79" s="53"/>
+      <x:c r="B79" s="62"/>
+      <x:c r="C79" s="53"/>
+      <x:c r="D79" s="58"/>
+      <x:c r="E79" s="59"/>
+      <x:c r="F79" s="53"/>
+      <x:c r="G79" s="58"/>
+      <x:c r="H79" s="60"/>
+      <x:c r="I79" s="63"/>
+      <x:c r="J79" s="63"/>
+      <x:c r="K79" s="63"/>
+      <x:c r="L79" s="63"/>
+      <x:c r="M79" s="63"/>
+      <x:c r="N79" s="63"/>
+      <x:c r="O79" s="63"/>
+      <x:c r="P79" s="63"/>
+    </x:row>
+    <x:row r="80" ht="38" customHeight="1">
+      <x:c r="A80" s="66"/>
+      <x:c r="B80" s="67"/>
+      <x:c r="C80" s="66"/>
+      <x:c r="D80" s="68"/>
+      <x:c r="E80" s="69"/>
+      <x:c r="F80" s="66"/>
+      <x:c r="G80" s="68"/>
+      <x:c r="H80" s="70"/>
+      <x:c r="I80" s="71"/>
+      <x:c r="J80" s="63"/>
+      <x:c r="K80" s="63"/>
+      <x:c r="L80" s="63"/>
+      <x:c r="M80" s="63"/>
+      <x:c r="N80" s="63"/>
+      <x:c r="O80" s="63"/>
+      <x:c r="P80" s="63"/>
+    </x:row>
+    <x:row r="81" ht="38" customHeight="1">
+      <x:c r="A81" s="53"/>
+      <x:c r="B81" s="62"/>
+      <x:c r="C81" s="53"/>
+      <x:c r="D81" s="58"/>
+      <x:c r="E81" s="59"/>
+      <x:c r="F81" s="53"/>
+      <x:c r="G81" s="58"/>
+      <x:c r="H81" s="60"/>
+      <x:c r="I81" s="63"/>
+      <x:c r="J81" s="63"/>
+      <x:c r="K81" s="63"/>
+      <x:c r="L81" s="63"/>
+      <x:c r="M81" s="63"/>
+      <x:c r="N81" s="63"/>
+      <x:c r="O81" s="63"/>
+      <x:c r="P81" s="63"/>
+    </x:row>
+    <x:row r="82" ht="38" customHeight="1">
+      <x:c r="A82" s="66"/>
+      <x:c r="B82" s="67"/>
+      <x:c r="C82" s="66"/>
+      <x:c r="D82" s="68"/>
+      <x:c r="E82" s="69"/>
+      <x:c r="F82" s="66"/>
+      <x:c r="G82" s="68"/>
+      <x:c r="H82" s="70"/>
+      <x:c r="I82" s="71"/>
+      <x:c r="J82" s="63"/>
+      <x:c r="K82" s="63"/>
+      <x:c r="L82" s="63"/>
+      <x:c r="M82" s="63"/>
+      <x:c r="N82" s="63"/>
+      <x:c r="O82" s="63"/>
+      <x:c r="P82" s="63"/>
+    </x:row>
+    <x:row r="83" ht="38" customHeight="1">
+      <x:c r="A83" s="53"/>
+      <x:c r="B83" s="62"/>
+      <x:c r="C83" s="53"/>
+      <x:c r="D83" s="58"/>
+      <x:c r="E83" s="59"/>
+      <x:c r="F83" s="53"/>
+      <x:c r="G83" s="58"/>
+      <x:c r="H83" s="60"/>
+      <x:c r="I83" s="63"/>
+      <x:c r="J83" s="63"/>
+      <x:c r="K83" s="63"/>
+      <x:c r="L83" s="63"/>
+      <x:c r="M83" s="63"/>
+      <x:c r="N83" s="63"/>
+      <x:c r="O83" s="63"/>
+      <x:c r="P83" s="63"/>
+    </x:row>
+    <x:row r="84" ht="38" customHeight="1">
+      <x:c r="A84" s="66"/>
+      <x:c r="B84" s="67"/>
+      <x:c r="C84" s="66"/>
+      <x:c r="D84" s="68"/>
+      <x:c r="E84" s="69"/>
+      <x:c r="F84" s="66"/>
+      <x:c r="G84" s="68"/>
+      <x:c r="H84" s="70"/>
+      <x:c r="I84" s="71"/>
+      <x:c r="J84" s="63"/>
+      <x:c r="K84" s="63"/>
+      <x:c r="L84" s="63"/>
+      <x:c r="M84" s="63"/>
+      <x:c r="N84" s="63"/>
+      <x:c r="O84" s="63"/>
+      <x:c r="P84" s="63"/>
+    </x:row>
+    <x:row r="85" ht="38" customHeight="1">
+      <x:c r="A85" s="53"/>
+      <x:c r="B85" s="62"/>
+      <x:c r="C85" s="53"/>
+      <x:c r="D85" s="58"/>
+      <x:c r="E85" s="59"/>
+      <x:c r="F85" s="53"/>
+      <x:c r="G85" s="58"/>
+      <x:c r="H85" s="60"/>
+      <x:c r="I85" s="63"/>
+      <x:c r="J85" s="63"/>
+      <x:c r="K85" s="63"/>
+      <x:c r="L85" s="63"/>
+      <x:c r="M85" s="63"/>
+      <x:c r="N85" s="63"/>
+      <x:c r="O85" s="63"/>
+      <x:c r="P85" s="63"/>
+    </x:row>
+    <x:row r="86" ht="38" customHeight="1">
+      <x:c r="A86" s="66"/>
+      <x:c r="B86" s="67"/>
+      <x:c r="C86" s="66"/>
+      <x:c r="D86" s="68"/>
+      <x:c r="E86" s="69"/>
+      <x:c r="F86" s="66"/>
+      <x:c r="G86" s="68"/>
+      <x:c r="H86" s="70"/>
+      <x:c r="I86" s="71"/>
+      <x:c r="J86" s="63"/>
+      <x:c r="K86" s="63"/>
+      <x:c r="L86" s="63"/>
+      <x:c r="M86" s="63"/>
+      <x:c r="N86" s="63"/>
+      <x:c r="O86" s="63"/>
+      <x:c r="P86" s="63"/>
+    </x:row>
+    <x:row r="87" ht="38" customHeight="1">
+      <x:c r="A87" s="53"/>
+      <x:c r="B87" s="62"/>
+      <x:c r="C87" s="53"/>
+      <x:c r="D87" s="58"/>
+      <x:c r="E87" s="59"/>
+      <x:c r="F87" s="53"/>
+      <x:c r="G87" s="58"/>
+      <x:c r="H87" s="60"/>
+      <x:c r="I87" s="63"/>
+      <x:c r="J87" s="63"/>
+      <x:c r="K87" s="63"/>
+      <x:c r="L87" s="63"/>
+      <x:c r="M87" s="63"/>
+      <x:c r="N87" s="63"/>
+      <x:c r="O87" s="63"/>
+      <x:c r="P87" s="63"/>
+    </x:row>
+    <x:row r="88" ht="38" customHeight="1">
+      <x:c r="A88" s="66"/>
+      <x:c r="B88" s="67"/>
+      <x:c r="C88" s="66"/>
+      <x:c r="D88" s="68"/>
+      <x:c r="E88" s="69"/>
+      <x:c r="F88" s="66"/>
+      <x:c r="G88" s="68"/>
+      <x:c r="H88" s="70"/>
+      <x:c r="I88" s="71"/>
+      <x:c r="J88" s="63"/>
+      <x:c r="K88" s="63"/>
+      <x:c r="L88" s="63"/>
+      <x:c r="M88" s="63"/>
+      <x:c r="N88" s="63"/>
+      <x:c r="O88" s="63"/>
+      <x:c r="P88" s="63"/>
+    </x:row>
+    <x:row r="89" ht="38" customHeight="1">
+      <x:c r="A89" s="53"/>
+      <x:c r="B89" s="62"/>
+      <x:c r="C89" s="53"/>
+      <x:c r="D89" s="58"/>
+      <x:c r="E89" s="59"/>
+      <x:c r="F89" s="53"/>
+      <x:c r="G89" s="58"/>
+      <x:c r="H89" s="60"/>
+      <x:c r="I89" s="63"/>
+      <x:c r="J89" s="63"/>
+      <x:c r="K89" s="63"/>
+      <x:c r="L89" s="63"/>
+      <x:c r="M89" s="63"/>
+      <x:c r="N89" s="63"/>
+      <x:c r="O89" s="63"/>
+      <x:c r="P89" s="63"/>
+    </x:row>
+    <x:row r="90" ht="38" customHeight="1">
+      <x:c r="A90" s="66"/>
+      <x:c r="B90" s="67"/>
+      <x:c r="C90" s="66"/>
+      <x:c r="D90" s="68"/>
+      <x:c r="E90" s="69"/>
+      <x:c r="F90" s="66"/>
+      <x:c r="G90" s="68"/>
+      <x:c r="H90" s="70"/>
+      <x:c r="I90" s="71"/>
+      <x:c r="J90" s="63"/>
+      <x:c r="K90" s="63"/>
+      <x:c r="L90" s="63"/>
+      <x:c r="M90" s="63"/>
+      <x:c r="N90" s="63"/>
+      <x:c r="O90" s="63"/>
+      <x:c r="P90" s="63"/>
+    </x:row>
+    <x:row r="91" ht="38" customHeight="1">
+      <x:c r="A91" s="53"/>
+      <x:c r="B91" s="62"/>
+      <x:c r="C91" s="53"/>
+      <x:c r="D91" s="58"/>
+      <x:c r="E91" s="59"/>
+      <x:c r="F91" s="53"/>
+      <x:c r="G91" s="58"/>
+      <x:c r="H91" s="60"/>
+      <x:c r="I91" s="63"/>
+      <x:c r="J91" s="63"/>
+      <x:c r="K91" s="63"/>
+      <x:c r="L91" s="63"/>
+      <x:c r="M91" s="63"/>
+      <x:c r="N91" s="63"/>
+      <x:c r="O91" s="63"/>
+      <x:c r="P91" s="63"/>
+    </x:row>
+    <x:row r="92" ht="38" customHeight="1">
+      <x:c r="A92" s="66"/>
+      <x:c r="B92" s="67"/>
+      <x:c r="C92" s="66"/>
+      <x:c r="D92" s="68"/>
+      <x:c r="E92" s="69"/>
+      <x:c r="F92" s="66"/>
+      <x:c r="G92" s="68"/>
+      <x:c r="H92" s="70"/>
+      <x:c r="I92" s="71"/>
+      <x:c r="J92" s="63"/>
+      <x:c r="K92" s="63"/>
+      <x:c r="L92" s="63"/>
+      <x:c r="M92" s="63"/>
+      <x:c r="N92" s="63"/>
+      <x:c r="O92" s="63"/>
+      <x:c r="P92" s="63"/>
+    </x:row>
+    <x:row r="93" ht="38" customHeight="1">
+      <x:c r="A93" s="53"/>
+      <x:c r="B93" s="62"/>
+      <x:c r="C93" s="53"/>
+      <x:c r="D93" s="58"/>
+      <x:c r="E93" s="59"/>
+      <x:c r="F93" s="53"/>
+      <x:c r="G93" s="58"/>
+      <x:c r="H93" s="60"/>
+      <x:c r="I93" s="63"/>
+      <x:c r="J93" s="63"/>
+      <x:c r="K93" s="63"/>
+      <x:c r="L93" s="63"/>
+      <x:c r="M93" s="63"/>
+      <x:c r="N93" s="63"/>
+      <x:c r="O93" s="63"/>
+      <x:c r="P93" s="63"/>
+    </x:row>
+    <x:row r="94" ht="38" customHeight="1">
+      <x:c r="A94" s="66"/>
+      <x:c r="B94" s="67"/>
+      <x:c r="C94" s="66"/>
+      <x:c r="D94" s="68"/>
+      <x:c r="E94" s="69"/>
+      <x:c r="F94" s="66"/>
+      <x:c r="G94" s="68"/>
+      <x:c r="H94" s="70"/>
+      <x:c r="I94" s="71"/>
+      <x:c r="J94" s="63"/>
+      <x:c r="K94" s="63"/>
+      <x:c r="L94" s="63"/>
+      <x:c r="M94" s="63"/>
+      <x:c r="N94" s="63"/>
+      <x:c r="O94" s="63"/>
+      <x:c r="P94" s="63"/>
+    </x:row>
+    <x:row r="95" ht="38" customHeight="1">
+      <x:c r="A95" s="53"/>
+      <x:c r="B95" s="62"/>
+      <x:c r="C95" s="53"/>
+      <x:c r="D95" s="58"/>
+      <x:c r="E95" s="59"/>
+      <x:c r="F95" s="53"/>
+      <x:c r="G95" s="58"/>
+      <x:c r="H95" s="60"/>
+      <x:c r="I95" s="63"/>
+      <x:c r="J95" s="63"/>
+      <x:c r="K95" s="63"/>
+      <x:c r="L95" s="63"/>
+      <x:c r="M95" s="63"/>
+      <x:c r="N95" s="63"/>
+      <x:c r="O95" s="63"/>
+      <x:c r="P95" s="63"/>
+    </x:row>
+    <x:row r="96" ht="38" customHeight="1">
+      <x:c r="A96" s="66"/>
+      <x:c r="B96" s="67"/>
+      <x:c r="C96" s="66"/>
+      <x:c r="D96" s="68"/>
+      <x:c r="E96" s="69"/>
+      <x:c r="F96" s="66"/>
+      <x:c r="G96" s="68"/>
+      <x:c r="H96" s="70"/>
+      <x:c r="I96" s="71"/>
+      <x:c r="J96" s="63"/>
+      <x:c r="K96" s="63"/>
+      <x:c r="L96" s="63"/>
+      <x:c r="M96" s="63"/>
+      <x:c r="N96" s="63"/>
+      <x:c r="O96" s="63"/>
+      <x:c r="P96" s="63"/>
+    </x:row>
+    <x:row r="97" ht="38" customHeight="1">
+      <x:c r="A97" s="53"/>
+      <x:c r="B97" s="62"/>
+      <x:c r="C97" s="53"/>
+      <x:c r="D97" s="58"/>
+      <x:c r="E97" s="59"/>
+      <x:c r="F97" s="53"/>
+      <x:c r="G97" s="58"/>
+      <x:c r="H97" s="60"/>
+      <x:c r="I97" s="63"/>
+      <x:c r="J97" s="63"/>
+      <x:c r="K97" s="63"/>
+      <x:c r="L97" s="63"/>
+      <x:c r="M97" s="63"/>
+      <x:c r="N97" s="63"/>
+      <x:c r="O97" s="63"/>
+      <x:c r="P97" s="63"/>
+    </x:row>
+    <x:row r="98" ht="38" customHeight="1">
+      <x:c r="A98" s="66"/>
+      <x:c r="B98" s="67"/>
+      <x:c r="C98" s="66"/>
+      <x:c r="D98" s="68"/>
+      <x:c r="E98" s="69"/>
+      <x:c r="F98" s="66"/>
+      <x:c r="G98" s="68"/>
+      <x:c r="H98" s="70"/>
+      <x:c r="I98" s="71"/>
+      <x:c r="J98" s="63"/>
+      <x:c r="K98" s="63"/>
+      <x:c r="L98" s="63"/>
+      <x:c r="M98" s="63"/>
+      <x:c r="N98" s="63"/>
+      <x:c r="O98" s="63"/>
+      <x:c r="P98" s="63"/>
+    </x:row>
+    <x:row r="99" ht="38" customHeight="1">
+      <x:c r="A99" s="53"/>
+      <x:c r="B99" s="62"/>
+      <x:c r="C99" s="53"/>
+      <x:c r="D99" s="58"/>
+      <x:c r="E99" s="59"/>
+      <x:c r="F99" s="53"/>
+      <x:c r="G99" s="58"/>
+      <x:c r="H99" s="60"/>
+      <x:c r="I99" s="63"/>
+      <x:c r="J99" s="63"/>
+      <x:c r="K99" s="63"/>
+      <x:c r="L99" s="63"/>
+      <x:c r="M99" s="63"/>
+      <x:c r="N99" s="63"/>
+      <x:c r="O99" s="63"/>
+      <x:c r="P99" s="63"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A2:P2"/>
+    <x:mergeCell ref="A4:P4"/>
+    <x:mergeCell ref="A5:P5"/>
+    <x:mergeCell ref="A17:P17"/>
+  </x:mergeCells>
+  <x:dataValidations count="5">
+    <x:dataValidation type="list" sqref="B3">
+      <x:formula1>"全部,定价与期限,位置与趋势,波动与形态,成交与活跃,持仓与结构,盘口与规模"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E3">
+      <x:formula1>"1,2,3,4,5,6,7,8"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="A7:A14">
+      <x:formula1>"期现,跨期,跨指数"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="D7:D14">
+      <x:formula1>"期货价,基差bp,年化"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E7:E14">
+      <x:formula1>"盘中优先,日终,历史日"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>